<commit_message>
feat: update player statistics and add new player to the data set
</commit_message>
<xml_diff>
--- a/Pontuação 2026.xlsx
+++ b/Pontuação 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luan-\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268D0D30-F7F1-4714-AAF8-20AE2C7F6FA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0F8751-E65A-4C0B-B188-230FDED1502F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="41">
   <si>
     <t>Atletas</t>
   </si>
@@ -144,9 +144,6 @@
   </si>
   <si>
     <t>João</t>
-  </si>
-  <si>
-    <t>Edgar</t>
   </si>
 </sst>
 </file>
@@ -4556,20 +4553,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43A1E9A1-0650-4526-8818-93833A813349}">
-  <dimension ref="B1:BJ41"/>
+  <dimension ref="B1:BJ40"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="1.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="18.140625" style="1" customWidth="1"/>
     <col min="4" max="7" width="7.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="21" width="6.7109375" style="1" hidden="1" customWidth="1"/>
-    <col min="22" max="22" width="7" style="1" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.28515625" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="13" width="6.28515625" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="5.28515625" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="18" width="6.28515625" style="1" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="6" style="1" hidden="1" customWidth="1"/>
+    <col min="20" max="22" width="7" style="1" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="5.5703125" style="1" hidden="1" customWidth="1"/>
+    <col min="24" max="26" width="6.5703125" style="1" hidden="1" customWidth="1"/>
+    <col min="27" max="28" width="5.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="29" max="29" width="6.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="30" max="31" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="5.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="33" max="35" width="6.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="4.5703125" style="1" hidden="1" customWidth="1"/>
@@ -4892,28 +4894,28 @@
         <v>40</v>
       </c>
       <c r="C4" s="6">
-        <f t="shared" ref="C4:C17" si="2">SUM(I4:BI4)</f>
-        <v>50</v>
+        <f>SUM(I4:BI4)</f>
+        <v>53</v>
       </c>
       <c r="D4" s="11">
-        <f t="shared" ref="D4:D17" si="3">SUM(I4:V4)</f>
+        <f>SUM(I4:V4)</f>
         <v>29</v>
       </c>
       <c r="E4" s="11">
-        <f t="shared" ref="E4:E17" si="4">SUM(W4:AI4)</f>
-        <v>21</v>
+        <f>SUM(W4:AI4)</f>
+        <v>24</v>
       </c>
       <c r="F4" s="11">
-        <f t="shared" ref="F4:F17" si="5">SUM(AJ4:AV4)</f>
+        <f>SUM(AJ4:AV4)</f>
         <v>0</v>
       </c>
       <c r="G4" s="11">
-        <f t="shared" ref="G4:G17" si="6">SUM(AW4:BI4)</f>
+        <f>SUM(AW4:BI4)</f>
         <v>0</v>
       </c>
       <c r="H4" s="11">
-        <f t="shared" ref="H4:H17" si="7">COUNT(I4:BI4)</f>
-        <v>22</v>
+        <f>COUNT(I4:BI4)</f>
+        <v>23</v>
       </c>
       <c r="I4" s="3">
         <v>3</v>
@@ -4993,7 +4995,9 @@
       <c r="AH4" s="3">
         <v>3</v>
       </c>
-      <c r="AI4" s="3"/>
+      <c r="AI4" s="3">
+        <v>3</v>
+      </c>
       <c r="AJ4" s="3"/>
       <c r="AK4" s="3"/>
       <c r="AL4" s="3"/>
@@ -5023,31 +5027,31 @@
     </row>
     <row r="5" spans="2:61" ht="14.1" customHeight="1">
       <c r="B5" s="14" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C5" s="6">
-        <f t="shared" si="2"/>
-        <v>34</v>
+        <f>SUM(I5:BI5)</f>
+        <v>37</v>
       </c>
       <c r="D5" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I5:V5)</f>
         <v>16</v>
       </c>
       <c r="E5" s="11">
-        <f t="shared" si="4"/>
-        <v>18</v>
+        <f>SUM(W5:AI5)</f>
+        <v>21</v>
       </c>
       <c r="F5" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ5:AV5)</f>
         <v>0</v>
       </c>
       <c r="G5" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW5:BI5)</f>
         <v>0</v>
       </c>
       <c r="H5" s="11">
-        <f t="shared" si="7"/>
-        <v>21</v>
+        <f>COUNT(I5:BI5)</f>
+        <v>23</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>19</v>
@@ -5062,16 +5066,16 @@
         <v>0</v>
       </c>
       <c r="M5" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N5" s="3">
-        <v>3</v>
-      </c>
-      <c r="O5" s="3">
-        <v>0</v>
-      </c>
-      <c r="P5" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Q5" s="3">
         <v>0</v>
@@ -5080,7 +5084,7 @@
         <v>0</v>
       </c>
       <c r="S5" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T5" s="3">
         <v>3</v>
@@ -5089,45 +5093,47 @@
         <v>3</v>
       </c>
       <c r="V5" s="3">
-        <v>3</v>
-      </c>
-      <c r="W5" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="W5" s="3">
+        <v>3</v>
       </c>
       <c r="X5" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y5" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>0</v>
       </c>
       <c r="Z5" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA5" s="3">
         <v>3</v>
       </c>
-      <c r="AB5" s="3">
-        <v>3</v>
+      <c r="AB5" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AC5" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE5" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="AD5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="3">
+        <v>3</v>
       </c>
       <c r="AF5" s="3">
         <v>3</v>
       </c>
       <c r="AG5" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AH5" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI5" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="AI5" s="3">
+        <v>3</v>
+      </c>
       <c r="AJ5" s="3"/>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
@@ -5157,30 +5163,30 @@
     </row>
     <row r="6" spans="2:61" ht="14.1" customHeight="1">
       <c r="B6" s="14" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="C6" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I6:BI6)</f>
         <v>34</v>
       </c>
       <c r="D6" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I6:V6)</f>
         <v>16</v>
       </c>
       <c r="E6" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W6:AI6)</f>
         <v>18</v>
       </c>
       <c r="F6" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ6:AV6)</f>
         <v>0</v>
       </c>
       <c r="G6" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW6:BI6)</f>
         <v>0</v>
       </c>
       <c r="H6" s="11">
-        <f t="shared" si="7"/>
+        <f>COUNT(I6:BI6)</f>
         <v>22</v>
       </c>
       <c r="I6" s="3" t="s">
@@ -5196,16 +5202,16 @@
         <v>0</v>
       </c>
       <c r="M6" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N6" s="3">
-        <v>0</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="O6" s="3">
+        <v>0</v>
+      </c>
+      <c r="P6" s="3">
+        <v>0</v>
       </c>
       <c r="Q6" s="3">
         <v>0</v>
@@ -5214,7 +5220,7 @@
         <v>0</v>
       </c>
       <c r="S6" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T6" s="3">
         <v>3</v>
@@ -5223,45 +5229,47 @@
         <v>3</v>
       </c>
       <c r="V6" s="3">
-        <v>0</v>
-      </c>
-      <c r="W6" s="3">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="X6" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y6" s="3">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Z6" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA6" s="3">
         <v>3</v>
       </c>
-      <c r="AB6" s="3" t="s">
-        <v>19</v>
+      <c r="AB6" s="3">
+        <v>3</v>
       </c>
       <c r="AC6" s="3">
-        <v>3</v>
-      </c>
-      <c r="AD6" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE6" s="3">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="AD6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE6" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AF6" s="3">
         <v>3</v>
       </c>
       <c r="AG6" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AH6" s="3">
-        <v>3</v>
-      </c>
-      <c r="AI6" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="AI6" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ6" s="3"/>
       <c r="AK6" s="3"/>
       <c r="AL6" s="3"/>
@@ -5294,28 +5302,28 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I7:BI7)</f>
         <v>32</v>
       </c>
       <c r="D7" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I7:V7)</f>
         <v>14</v>
       </c>
       <c r="E7" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W7:AI7)</f>
         <v>18</v>
       </c>
       <c r="F7" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ7:AV7)</f>
         <v>0</v>
       </c>
       <c r="G7" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW7:BI7)</f>
         <v>0</v>
       </c>
       <c r="H7" s="11">
-        <f t="shared" si="7"/>
-        <v>25</v>
+        <f>COUNT(I7:BI7)</f>
+        <v>26</v>
       </c>
       <c r="I7" s="3">
         <v>3</v>
@@ -5395,7 +5403,9 @@
       <c r="AH7" s="3">
         <v>3</v>
       </c>
-      <c r="AI7" s="3"/>
+      <c r="AI7" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ7" s="3"/>
       <c r="AK7" s="3"/>
       <c r="AL7" s="3"/>
@@ -5428,27 +5438,27 @@
         <v>36</v>
       </c>
       <c r="C8" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I8:BI8)</f>
         <v>29</v>
       </c>
       <c r="D8" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I8:V8)</f>
         <v>20</v>
       </c>
       <c r="E8" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W8:AI8)</f>
         <v>9</v>
       </c>
       <c r="F8" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ8:AV8)</f>
         <v>0</v>
       </c>
       <c r="G8" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW8:BI8)</f>
         <v>0</v>
       </c>
       <c r="H8" s="11">
-        <f t="shared" si="7"/>
+        <f>COUNT(I8:BI8)</f>
         <v>17</v>
       </c>
       <c r="I8" s="3" t="s">
@@ -5529,7 +5539,9 @@
       <c r="AH8" s="3">
         <v>0</v>
       </c>
-      <c r="AI8" s="3"/>
+      <c r="AI8" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ8" s="3"/>
       <c r="AK8" s="3"/>
       <c r="AL8" s="3"/>
@@ -5562,28 +5574,28 @@
         <v>18</v>
       </c>
       <c r="C9" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I9:BI9)</f>
         <v>28</v>
       </c>
       <c r="D9" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I9:V9)</f>
         <v>10</v>
       </c>
       <c r="E9" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W9:AI9)</f>
         <v>18</v>
       </c>
       <c r="F9" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ9:AV9)</f>
         <v>0</v>
       </c>
       <c r="G9" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW9:BI9)</f>
         <v>0</v>
       </c>
       <c r="H9" s="11">
-        <f t="shared" si="7"/>
-        <v>24</v>
+        <f>COUNT(I9:BI9)</f>
+        <v>25</v>
       </c>
       <c r="I9" s="3">
         <v>3</v>
@@ -5663,7 +5675,9 @@
       <c r="AH9" s="3">
         <v>0</v>
       </c>
-      <c r="AI9" s="3"/>
+      <c r="AI9" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ9" s="3"/>
       <c r="AK9" s="3"/>
       <c r="AL9" s="3"/>
@@ -5693,43 +5707,43 @@
     </row>
     <row r="10" spans="2:61" ht="14.1" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C10" s="6">
-        <f t="shared" si="2"/>
-        <v>26</v>
+        <f>SUM(I10:BI10)</f>
+        <v>28</v>
       </c>
       <c r="D10" s="11">
-        <f t="shared" si="3"/>
-        <v>17</v>
+        <f>SUM(I10:V10)</f>
+        <v>13</v>
       </c>
       <c r="E10" s="11">
-        <f t="shared" si="4"/>
-        <v>9</v>
+        <f>SUM(W10:AI10)</f>
+        <v>15</v>
       </c>
       <c r="F10" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ10:AV10)</f>
         <v>0</v>
       </c>
       <c r="G10" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW10:BI10)</f>
         <v>0</v>
       </c>
       <c r="H10" s="11">
-        <f t="shared" si="7"/>
-        <v>19</v>
-      </c>
-      <c r="I10" s="3">
-        <v>3</v>
+        <f>COUNT(I10:BI10)</f>
+        <v>15</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="J10" s="3">
         <v>3</v>
       </c>
-      <c r="K10" s="3">
-        <v>1</v>
-      </c>
-      <c r="L10" s="3">
-        <v>3</v>
+      <c r="K10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>19</v>
@@ -5749,8 +5763,8 @@
       <c r="R10" s="3">
         <v>3</v>
       </c>
-      <c r="S10" s="3" t="s">
-        <v>19</v>
+      <c r="S10" s="3">
+        <v>3</v>
       </c>
       <c r="T10" s="3">
         <v>0</v>
@@ -5767,37 +5781,39 @@
       <c r="X10" s="3">
         <v>3</v>
       </c>
-      <c r="Y10" s="3">
-        <v>0</v>
+      <c r="Y10" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Z10" s="3">
         <v>0</v>
       </c>
-      <c r="AA10" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="3">
-        <v>0</v>
+      <c r="AA10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB10" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AC10" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD10" s="3">
-        <v>3</v>
-      </c>
-      <c r="AE10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AF10" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="AD10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE10" s="3">
+        <v>3</v>
+      </c>
+      <c r="AF10" s="3">
+        <v>0</v>
       </c>
       <c r="AG10" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH10" s="3">
-        <v>3</v>
-      </c>
-      <c r="AI10" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="AH10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI10" s="3">
+        <v>3</v>
+      </c>
       <c r="AJ10" s="3"/>
       <c r="AK10" s="3"/>
       <c r="AL10" s="3"/>
@@ -5827,37 +5843,37 @@
     </row>
     <row r="11" spans="2:61" ht="14.1" customHeight="1">
       <c r="B11" s="14" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C11" s="6">
-        <f t="shared" si="2"/>
-        <v>25</v>
+        <f>SUM(I11:BI11)</f>
+        <v>26</v>
       </c>
       <c r="D11" s="11">
-        <f t="shared" si="3"/>
-        <v>16</v>
+        <f>SUM(I11:V11)</f>
+        <v>17</v>
       </c>
       <c r="E11" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W11:AI11)</f>
         <v>9</v>
       </c>
       <c r="F11" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ11:AV11)</f>
         <v>0</v>
       </c>
       <c r="G11" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW11:BI11)</f>
         <v>0</v>
       </c>
       <c r="H11" s="11">
-        <f t="shared" si="7"/>
-        <v>23</v>
+        <f>COUNT(I11:BI11)</f>
+        <v>19</v>
       </c>
       <c r="I11" s="3">
         <v>3</v>
       </c>
       <c r="J11" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K11" s="3">
         <v>1</v>
@@ -5865,73 +5881,75 @@
       <c r="L11" s="3">
         <v>3</v>
       </c>
-      <c r="M11" s="3">
-        <v>0</v>
-      </c>
-      <c r="N11" s="3">
-        <v>0</v>
-      </c>
-      <c r="O11" s="3">
-        <v>3</v>
+      <c r="M11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="P11" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="3" t="s">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="Q11" s="3">
+        <v>3</v>
       </c>
       <c r="R11" s="3">
-        <v>0</v>
-      </c>
-      <c r="S11" s="3">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="S11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="T11" s="3">
-        <v>3</v>
-      </c>
-      <c r="U11" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="U11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="V11" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W11" s="3">
         <v>0</v>
       </c>
       <c r="X11" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y11" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Z11" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="3">
         <v>0</v>
       </c>
-      <c r="AB11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AC11" s="3" t="s">
-        <v>19</v>
+      <c r="AB11" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="3">
+        <v>0</v>
       </c>
       <c r="AD11" s="3">
         <v>3</v>
       </c>
-      <c r="AE11" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF11" s="3">
-        <v>0</v>
+      <c r="AE11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AF11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AG11" s="3">
         <v>0</v>
       </c>
       <c r="AH11" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI11" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="AI11" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ11" s="3"/>
       <c r="AK11" s="3"/>
       <c r="AL11" s="3"/>
@@ -5961,43 +5979,43 @@
     </row>
     <row r="12" spans="2:61" ht="14.1" customHeight="1">
       <c r="B12" s="14" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C12" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I12:BI12)</f>
         <v>25</v>
       </c>
       <c r="D12" s="11">
-        <f t="shared" si="3"/>
-        <v>13</v>
+        <f>SUM(I12:V12)</f>
+        <v>16</v>
       </c>
       <c r="E12" s="11">
-        <f t="shared" si="4"/>
-        <v>12</v>
+        <f>SUM(W12:AI12)</f>
+        <v>9</v>
       </c>
       <c r="F12" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ12:AV12)</f>
         <v>0</v>
       </c>
       <c r="G12" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW12:BI12)</f>
         <v>0</v>
       </c>
       <c r="H12" s="11">
-        <f t="shared" si="7"/>
-        <v>20</v>
+        <f>COUNT(I12:BI12)</f>
+        <v>24</v>
       </c>
       <c r="I12" s="3">
-        <v>0</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
       </c>
       <c r="K12" s="3">
         <v>1</v>
       </c>
       <c r="L12" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M12" s="3">
         <v>0</v>
@@ -6008,53 +6026,53 @@
       <c r="O12" s="3">
         <v>3</v>
       </c>
-      <c r="P12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>3</v>
+      <c r="P12" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="R12" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S12" s="3">
         <v>0</v>
       </c>
       <c r="T12" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U12" s="3">
-        <v>3</v>
-      </c>
-      <c r="V12" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="V12" s="3">
+        <v>3</v>
       </c>
       <c r="W12" s="3">
         <v>0</v>
       </c>
       <c r="X12" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Z12" s="3">
         <v>3</v>
       </c>
       <c r="AA12" s="3">
-        <v>3</v>
-      </c>
-      <c r="AB12" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="AB12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AC12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AD12" s="3" t="s">
-        <v>19</v>
+      <c r="AD12" s="3">
+        <v>3</v>
       </c>
       <c r="AE12" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AF12" s="3">
         <v>0</v>
@@ -6062,10 +6080,12 @@
       <c r="AG12" s="3">
         <v>0</v>
       </c>
-      <c r="AH12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI12" s="3"/>
+      <c r="AH12" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI12" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ12" s="3"/>
       <c r="AK12" s="3"/>
       <c r="AL12" s="3"/>
@@ -6095,37 +6115,37 @@
     </row>
     <row r="13" spans="2:61" ht="14.1" customHeight="1">
       <c r="B13" s="14" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C13" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I13:BI13)</f>
         <v>25</v>
       </c>
       <c r="D13" s="11">
-        <f t="shared" si="3"/>
-        <v>10</v>
+        <f>SUM(I13:V13)</f>
+        <v>13</v>
       </c>
       <c r="E13" s="11">
-        <f t="shared" si="4"/>
-        <v>15</v>
+        <f>SUM(W13:AI13)</f>
+        <v>12</v>
       </c>
       <c r="F13" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ13:AV13)</f>
         <v>0</v>
       </c>
       <c r="G13" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW13:BI13)</f>
         <v>0</v>
       </c>
       <c r="H13" s="11">
-        <f t="shared" si="7"/>
-        <v>22</v>
+        <f>COUNT(I13:BI13)</f>
+        <v>21</v>
       </c>
       <c r="I13" s="3">
         <v>0</v>
       </c>
-      <c r="J13" s="3">
-        <v>0</v>
+      <c r="J13" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="K13" s="3">
         <v>1</v>
@@ -6145,61 +6165,63 @@
       <c r="P13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Q13" s="3" t="s">
-        <v>19</v>
+      <c r="Q13" s="3">
+        <v>3</v>
       </c>
       <c r="R13" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S13" s="3">
         <v>0</v>
       </c>
       <c r="T13" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U13" s="3">
-        <v>0</v>
-      </c>
-      <c r="V13" s="3">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="V13" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="W13" s="3">
         <v>0</v>
       </c>
       <c r="X13" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y13" s="3">
-        <v>3</v>
-      </c>
-      <c r="Z13" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="Z13" s="3">
+        <v>3</v>
       </c>
       <c r="AA13" s="3">
         <v>3</v>
       </c>
       <c r="AB13" s="3">
-        <v>3</v>
-      </c>
-      <c r="AC13" s="3">
-        <v>3</v>
-      </c>
-      <c r="AD13" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE13" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="AC13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE13" s="3">
+        <v>3</v>
       </c>
       <c r="AF13" s="3">
         <v>0</v>
       </c>
       <c r="AG13" s="3">
-        <v>3</v>
-      </c>
-      <c r="AH13" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI13" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="AH13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI13" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ13" s="3"/>
       <c r="AK13" s="3"/>
       <c r="AL13" s="3"/>
@@ -6229,100 +6251,100 @@
     </row>
     <row r="14" spans="2:61" ht="14.1" customHeight="1">
       <c r="B14" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="6">
+        <f>SUM(I14:BI14)</f>
+        <v>25</v>
+      </c>
+      <c r="D14" s="11">
+        <f>SUM(I14:V14)</f>
+        <v>10</v>
+      </c>
+      <c r="E14" s="11">
+        <f>SUM(W14:AI14)</f>
         <v>15</v>
       </c>
-      <c r="C14" s="6">
-        <f t="shared" si="2"/>
-        <v>25</v>
-      </c>
-      <c r="D14" s="11">
-        <f t="shared" si="3"/>
-        <v>13</v>
-      </c>
-      <c r="E14" s="11">
-        <f t="shared" si="4"/>
-        <v>12</v>
-      </c>
       <c r="F14" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ14:AV14)</f>
         <v>0</v>
       </c>
       <c r="G14" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW14:BI14)</f>
         <v>0</v>
       </c>
       <c r="H14" s="11">
-        <f t="shared" si="7"/>
-        <v>14</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>19</v>
+        <f>COUNT(I14:BI14)</f>
+        <v>23</v>
+      </c>
+      <c r="I14" s="3">
+        <v>0</v>
       </c>
       <c r="J14" s="3">
-        <v>3</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P14" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="3">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="K14" s="3">
+        <v>1</v>
+      </c>
+      <c r="L14" s="3">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3">
+        <v>0</v>
+      </c>
+      <c r="N14" s="3">
+        <v>0</v>
+      </c>
+      <c r="O14" s="3">
+        <v>3</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="R14" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S14" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T14" s="3">
-        <v>0</v>
-      </c>
-      <c r="U14" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="U14" s="3">
+        <v>0</v>
       </c>
       <c r="V14" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W14" s="3">
         <v>0</v>
       </c>
       <c r="X14" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z14" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB14" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="Y14" s="3">
+        <v>3</v>
+      </c>
+      <c r="Z14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA14" s="3">
+        <v>3</v>
+      </c>
+      <c r="AB14" s="3">
+        <v>3</v>
       </c>
       <c r="AC14" s="3">
         <v>3</v>
       </c>
-      <c r="AD14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE14" s="3">
-        <v>3</v>
+      <c r="AD14" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AF14" s="3">
         <v>0</v>
@@ -6330,10 +6352,12 @@
       <c r="AG14" s="3">
         <v>3</v>
       </c>
-      <c r="AH14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI14" s="3"/>
+      <c r="AH14" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ14" s="3"/>
       <c r="AK14" s="3"/>
       <c r="AL14" s="3"/>
@@ -6366,27 +6390,27 @@
         <v>6</v>
       </c>
       <c r="C15" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I15:BI15)</f>
         <v>21</v>
       </c>
       <c r="D15" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I15:V15)</f>
         <v>9</v>
       </c>
       <c r="E15" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W15:AI15)</f>
         <v>12</v>
       </c>
       <c r="F15" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ15:AV15)</f>
         <v>0</v>
       </c>
       <c r="G15" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW15:BI15)</f>
         <v>0</v>
       </c>
       <c r="H15" s="11">
-        <f t="shared" si="7"/>
+        <f>COUNT(I15:BI15)</f>
         <v>17</v>
       </c>
       <c r="I15" s="3">
@@ -6467,7 +6491,9 @@
       <c r="AH15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AI15" s="3"/>
+      <c r="AI15" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ15" s="3"/>
       <c r="AK15" s="3"/>
       <c r="AL15" s="3"/>
@@ -6500,28 +6526,28 @@
         <v>17</v>
       </c>
       <c r="C16" s="6">
-        <f t="shared" si="2"/>
-        <v>6</v>
+        <f>SUM(I16:BI16)</f>
+        <v>9</v>
       </c>
       <c r="D16" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I16:V16)</f>
         <v>0</v>
       </c>
       <c r="E16" s="11">
-        <f t="shared" si="4"/>
-        <v>6</v>
+        <f>SUM(W16:AI16)</f>
+        <v>9</v>
       </c>
       <c r="F16" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ16:AV16)</f>
         <v>0</v>
       </c>
       <c r="G16" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW16:BI16)</f>
         <v>0</v>
       </c>
       <c r="H16" s="11">
-        <f t="shared" si="7"/>
-        <v>2</v>
+        <f>COUNT(I16:BI16)</f>
+        <v>3</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>19</v>
@@ -6601,7 +6627,9 @@
       <c r="AH16" s="3">
         <v>3</v>
       </c>
-      <c r="AI16" s="3"/>
+      <c r="AI16" s="3">
+        <v>3</v>
+      </c>
       <c r="AJ16" s="3"/>
       <c r="AK16" s="3"/>
       <c r="AL16" s="3"/>
@@ -6634,27 +6662,27 @@
         <v>10</v>
       </c>
       <c r="C17" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I17:BI17)</f>
         <v>1</v>
       </c>
       <c r="D17" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I17:V17)</f>
         <v>1</v>
       </c>
       <c r="E17" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W17:AI17)</f>
         <v>0</v>
       </c>
       <c r="F17" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ17:AV17)</f>
         <v>0</v>
       </c>
       <c r="G17" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW17:BI17)</f>
         <v>0</v>
       </c>
       <c r="H17" s="11">
-        <f t="shared" si="7"/>
+        <f>COUNT(I17:BI17)</f>
         <v>2</v>
       </c>
       <c r="I17" s="3" t="s">
@@ -6735,7 +6763,9 @@
       <c r="AH17" s="3">
         <v>0</v>
       </c>
-      <c r="AI17" s="3"/>
+      <c r="AI17" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
       <c r="AL17" s="3"/>
@@ -6789,27 +6819,27 @@
         <v>46025</v>
       </c>
       <c r="J18" s="5">
-        <f t="shared" ref="J18:O18" si="8">I18+7</f>
+        <f t="shared" ref="J18:O18" si="2">I18+7</f>
         <v>46032</v>
       </c>
       <c r="K18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46039</v>
       </c>
       <c r="L18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46046</v>
       </c>
       <c r="M18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46053</v>
       </c>
       <c r="N18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46060</v>
       </c>
       <c r="O18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46067</v>
       </c>
       <c r="P18" s="5">
@@ -6840,159 +6870,159 @@
         <v>46109</v>
       </c>
       <c r="W18" s="5">
-        <f t="shared" ref="W18:BH18" si="9">V18+7</f>
+        <f t="shared" ref="W18:BH18" si="3">V18+7</f>
         <v>46116</v>
       </c>
       <c r="X18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46123</v>
       </c>
       <c r="Y18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46130</v>
       </c>
       <c r="Z18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46137</v>
       </c>
       <c r="AA18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46144</v>
       </c>
       <c r="AB18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46151</v>
       </c>
       <c r="AC18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46158</v>
       </c>
       <c r="AD18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46165</v>
       </c>
       <c r="AE18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46172</v>
       </c>
       <c r="AF18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46179</v>
       </c>
       <c r="AG18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46186</v>
       </c>
       <c r="AH18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46193</v>
       </c>
       <c r="AI18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46200</v>
       </c>
       <c r="AJ18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46207</v>
       </c>
       <c r="AK18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46214</v>
       </c>
       <c r="AL18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46221</v>
       </c>
       <c r="AM18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46228</v>
       </c>
       <c r="AN18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46235</v>
       </c>
       <c r="AO18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46242</v>
       </c>
       <c r="AP18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46249</v>
       </c>
       <c r="AQ18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46256</v>
       </c>
       <c r="AR18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46263</v>
       </c>
       <c r="AS18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46270</v>
       </c>
       <c r="AT18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46277</v>
       </c>
       <c r="AU18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46284</v>
       </c>
       <c r="AV18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46291</v>
       </c>
       <c r="AW18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46298</v>
       </c>
       <c r="AX18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46305</v>
       </c>
       <c r="AY18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46312</v>
       </c>
       <c r="AZ18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46319</v>
       </c>
       <c r="BA18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46326</v>
       </c>
       <c r="BB18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46333</v>
       </c>
       <c r="BC18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46340</v>
       </c>
       <c r="BD18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46347</v>
       </c>
       <c r="BE18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46354</v>
       </c>
       <c r="BF18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46361</v>
       </c>
       <c r="BG18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46368</v>
       </c>
       <c r="BH18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46375</v>
       </c>
       <c r="BI18" s="5">
-        <f t="shared" ref="BI18" si="10">BH18+7</f>
+        <f t="shared" ref="BI18" si="4">BH18+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -7002,7 +7032,7 @@
       </c>
       <c r="C19" s="6">
         <f>SUM(I19:BI19)</f>
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D19" s="11">
         <f>SUM(I19:V19)</f>
@@ -7010,7 +7040,7 @@
       </c>
       <c r="E19" s="11">
         <f>SUM(W19:AI19)</f>
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F19" s="11">
         <f>SUM(AJ19:AV19)</f>
@@ -7022,7 +7052,7 @@
       </c>
       <c r="H19" s="11">
         <f>COUNT(I19:BI19)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I19" s="3">
         <v>3</v>
@@ -7102,7 +7132,9 @@
       <c r="AH19" s="3">
         <v>0</v>
       </c>
-      <c r="AI19" s="3"/>
+      <c r="AI19" s="3">
+        <v>3</v>
+      </c>
       <c r="AJ19" s="3"/>
       <c r="AK19" s="3"/>
       <c r="AL19" s="3"/>
@@ -7156,7 +7188,7 @@
       </c>
       <c r="H20" s="11">
         <f>COUNT(I20:BI20)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>19</v>
@@ -7167,8 +7199,8 @@
       <c r="K20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="L20" s="3" t="s">
-        <v>19</v>
+      <c r="L20" s="3">
+        <v>0</v>
       </c>
       <c r="M20" s="3">
         <v>3</v>
@@ -7236,7 +7268,9 @@
       <c r="AH20" s="3">
         <v>0</v>
       </c>
-      <c r="AI20" s="3"/>
+      <c r="AI20" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
       <c r="AL20" s="3"/>
@@ -7358,23 +7392,23 @@
         <v>46032</v>
       </c>
       <c r="K23" s="5">
-        <f t="shared" ref="K23:BH23" si="11">J23+7</f>
+        <f t="shared" ref="K23:BH23" si="5">J23+7</f>
         <v>46039</v>
       </c>
       <c r="L23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46046</v>
       </c>
       <c r="M23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46053</v>
       </c>
       <c r="N23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46060</v>
       </c>
       <c r="O23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46067</v>
       </c>
       <c r="P23" s="5">
@@ -7385,179 +7419,179 @@
         <v>46074</v>
       </c>
       <c r="R23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46081</v>
       </c>
       <c r="S23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46088</v>
       </c>
       <c r="T23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46095</v>
       </c>
       <c r="U23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46102</v>
       </c>
       <c r="V23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46109</v>
       </c>
       <c r="W23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46116</v>
       </c>
       <c r="X23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46123</v>
       </c>
       <c r="Y23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46130</v>
       </c>
       <c r="Z23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46137</v>
       </c>
       <c r="AA23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46144</v>
       </c>
       <c r="AB23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46151</v>
       </c>
       <c r="AC23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46158</v>
       </c>
       <c r="AD23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46165</v>
       </c>
       <c r="AE23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46172</v>
       </c>
       <c r="AF23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46179</v>
       </c>
       <c r="AG23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46186</v>
       </c>
       <c r="AH23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46193</v>
       </c>
       <c r="AI23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46200</v>
       </c>
       <c r="AJ23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46207</v>
       </c>
       <c r="AK23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46214</v>
       </c>
       <c r="AL23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46221</v>
       </c>
       <c r="AM23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46228</v>
       </c>
       <c r="AN23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46235</v>
       </c>
       <c r="AO23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46242</v>
       </c>
       <c r="AP23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46249</v>
       </c>
       <c r="AQ23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46256</v>
       </c>
       <c r="AR23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46263</v>
       </c>
       <c r="AS23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46270</v>
       </c>
       <c r="AT23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46277</v>
       </c>
       <c r="AU23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46284</v>
       </c>
       <c r="AV23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46291</v>
       </c>
       <c r="AW23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46298</v>
       </c>
       <c r="AX23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46305</v>
       </c>
       <c r="AY23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46312</v>
       </c>
       <c r="AZ23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46319</v>
       </c>
       <c r="BA23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46326</v>
       </c>
       <c r="BB23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46333</v>
       </c>
       <c r="BC23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46340</v>
       </c>
       <c r="BD23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46347</v>
       </c>
       <c r="BE23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46354</v>
       </c>
       <c r="BF23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46361</v>
       </c>
       <c r="BG23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46368</v>
       </c>
       <c r="BH23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46375</v>
       </c>
       <c r="BI23" s="5">
-        <f t="shared" ref="BI23" si="12">BH23+7</f>
+        <f t="shared" ref="BI23" si="6">BH23+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -7566,28 +7600,28 @@
         <v>40</v>
       </c>
       <c r="C24" s="6">
-        <f t="shared" ref="C24:C38" si="13">SUM(I24:BI24)</f>
-        <v>43</v>
+        <f>SUM(I24:BI24)</f>
+        <v>44</v>
       </c>
       <c r="D24" s="11">
-        <f t="shared" ref="D24:D38" si="14">SUM(I24:V24)</f>
+        <f>SUM(I24:V24)</f>
         <v>20</v>
       </c>
       <c r="E24" s="11">
-        <f t="shared" ref="E24:E38" si="15">SUM(W24:AI24)</f>
+        <f>SUM(W24:AI24)</f>
+        <v>24</v>
+      </c>
+      <c r="F24" s="11">
+        <f>SUM(AJ24:AV24)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="11">
+        <f>SUM(AW24:BI24)</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="11">
+        <f>COUNT(I24:BI24)</f>
         <v>23</v>
-      </c>
-      <c r="F24" s="11">
-        <f t="shared" ref="F24:F38" si="16">SUM(AJ24:AV24)</f>
-        <v>0</v>
-      </c>
-      <c r="G24" s="11">
-        <f t="shared" ref="G24:G38" si="17">SUM(AW24:BI24)</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="11">
-        <f t="shared" ref="H24:H38" si="18">COUNT(I24:BI24)</f>
-        <v>22</v>
       </c>
       <c r="I24" s="3">
         <v>2</v>
@@ -7667,7 +7701,9 @@
       <c r="AH24" s="3">
         <v>2</v>
       </c>
-      <c r="AI24" s="3"/>
+      <c r="AI24" s="3">
+        <v>1</v>
+      </c>
       <c r="AJ24" s="3"/>
       <c r="AK24" s="3"/>
       <c r="AL24" s="3"/>
@@ -7700,28 +7736,28 @@
         <v>9</v>
       </c>
       <c r="C25" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I25:BI25)</f>
         <v>39</v>
       </c>
       <c r="D25" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I25:V25)</f>
         <v>22</v>
       </c>
       <c r="E25" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W25:AI25)</f>
         <v>17</v>
       </c>
       <c r="F25" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ25:AV25)</f>
         <v>0</v>
       </c>
       <c r="G25" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW25:BI25)</f>
         <v>0</v>
       </c>
       <c r="H25" s="11">
-        <f t="shared" si="18"/>
-        <v>23</v>
+        <f>COUNT(I25:BI25)</f>
+        <v>24</v>
       </c>
       <c r="I25" s="3">
         <v>0</v>
@@ -7801,7 +7837,9 @@
       <c r="AH25" s="3">
         <v>1</v>
       </c>
-      <c r="AI25" s="3"/>
+      <c r="AI25" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ25" s="3"/>
       <c r="AK25" s="3"/>
       <c r="AL25" s="3"/>
@@ -7834,28 +7872,28 @@
         <v>33</v>
       </c>
       <c r="C26" s="6">
-        <f t="shared" si="13"/>
-        <v>33</v>
+        <f>SUM(I26:BI26)</f>
+        <v>34</v>
       </c>
       <c r="D26" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I26:V26)</f>
         <v>19</v>
       </c>
       <c r="E26" s="11">
-        <f t="shared" si="15"/>
-        <v>14</v>
+        <f>SUM(W26:AI26)</f>
+        <v>15</v>
       </c>
       <c r="F26" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ26:AV26)</f>
         <v>0</v>
       </c>
       <c r="G26" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW26:BI26)</f>
         <v>0</v>
       </c>
       <c r="H26" s="11">
-        <f t="shared" si="18"/>
-        <v>21</v>
+        <f>COUNT(I26:BI26)</f>
+        <v>22</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>19</v>
@@ -7935,7 +7973,9 @@
       <c r="AH26" s="3">
         <v>1</v>
       </c>
-      <c r="AI26" s="3"/>
+      <c r="AI26" s="3">
+        <v>1</v>
+      </c>
       <c r="AJ26" s="3"/>
       <c r="AK26" s="3"/>
       <c r="AL26" s="3"/>
@@ -7968,28 +8008,28 @@
         <v>5</v>
       </c>
       <c r="C27" s="6">
-        <f t="shared" si="13"/>
-        <v>30</v>
+        <f>SUM(I27:BI27)</f>
+        <v>31</v>
       </c>
       <c r="D27" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I27:V27)</f>
         <v>19</v>
       </c>
       <c r="E27" s="11">
-        <f t="shared" si="15"/>
-        <v>11</v>
+        <f>SUM(W27:AI27)</f>
+        <v>12</v>
       </c>
       <c r="F27" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ27:AV27)</f>
         <v>0</v>
       </c>
       <c r="G27" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW27:BI27)</f>
         <v>0</v>
       </c>
       <c r="H27" s="11">
-        <f t="shared" si="18"/>
-        <v>22</v>
+        <f>COUNT(I27:BI27)</f>
+        <v>23</v>
       </c>
       <c r="I27" s="3">
         <v>4</v>
@@ -8069,7 +8109,9 @@
       <c r="AH27" s="3">
         <v>0</v>
       </c>
-      <c r="AI27" s="3"/>
+      <c r="AI27" s="3">
+        <v>1</v>
+      </c>
       <c r="AJ27" s="3"/>
       <c r="AK27" s="3"/>
       <c r="AL27" s="3"/>
@@ -8102,28 +8144,28 @@
         <v>11</v>
       </c>
       <c r="C28" s="6">
-        <f t="shared" si="13"/>
-        <v>27</v>
+        <f>SUM(I28:BI28)</f>
+        <v>28</v>
       </c>
       <c r="D28" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I28:V28)</f>
         <v>14</v>
       </c>
       <c r="E28" s="11">
-        <f t="shared" si="15"/>
-        <v>13</v>
+        <f>SUM(W28:AI28)</f>
+        <v>14</v>
       </c>
       <c r="F28" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ28:AV28)</f>
         <v>0</v>
       </c>
       <c r="G28" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW28:BI28)</f>
         <v>0</v>
       </c>
       <c r="H28" s="11">
-        <f t="shared" si="18"/>
-        <v>19</v>
+        <f>COUNT(I28:BI28)</f>
+        <v>20</v>
       </c>
       <c r="I28" s="3">
         <v>0</v>
@@ -8203,7 +8245,9 @@
       <c r="AH28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AI28" s="3"/>
+      <c r="AI28" s="3">
+        <v>1</v>
+      </c>
       <c r="AJ28" s="3"/>
       <c r="AK28" s="3"/>
       <c r="AL28" s="3"/>
@@ -8236,28 +8280,28 @@
         <v>3</v>
       </c>
       <c r="C29" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I29:BI29)</f>
         <v>27</v>
       </c>
       <c r="D29" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I29:V29)</f>
         <v>10</v>
       </c>
       <c r="E29" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W29:AI29)</f>
         <v>17</v>
       </c>
       <c r="F29" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ29:AV29)</f>
         <v>0</v>
       </c>
       <c r="G29" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW29:BI29)</f>
         <v>0</v>
       </c>
       <c r="H29" s="11">
-        <f t="shared" si="18"/>
-        <v>22</v>
+        <f>COUNT(I29:BI29)</f>
+        <v>23</v>
       </c>
       <c r="I29" s="3">
         <v>1</v>
@@ -8337,7 +8381,9 @@
       <c r="AH29" s="3">
         <v>2</v>
       </c>
-      <c r="AI29" s="3"/>
+      <c r="AI29" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ29" s="3"/>
       <c r="AK29" s="3"/>
       <c r="AL29" s="3"/>
@@ -8367,111 +8413,113 @@
     </row>
     <row r="30" spans="2:61" ht="14.1" customHeight="1">
       <c r="B30" s="14" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="C30" s="6">
-        <f t="shared" si="13"/>
-        <v>22</v>
+        <f>SUM(I30:BI30)</f>
+        <v>23</v>
       </c>
       <c r="D30" s="11">
-        <f t="shared" si="14"/>
-        <v>11</v>
+        <f>SUM(I30:V30)</f>
+        <v>13</v>
       </c>
       <c r="E30" s="11">
-        <f t="shared" si="15"/>
-        <v>11</v>
+        <f>SUM(W30:AI30)</f>
+        <v>10</v>
       </c>
       <c r="F30" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ30:AV30)</f>
         <v>0</v>
       </c>
       <c r="G30" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW30:BI30)</f>
         <v>0</v>
       </c>
       <c r="H30" s="11">
-        <f t="shared" si="18"/>
-        <v>12</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>19</v>
+        <f>COUNT(I30:BI30)</f>
+        <v>25</v>
+      </c>
+      <c r="I30" s="3">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3">
+        <v>0</v>
       </c>
       <c r="K30" s="3">
+        <v>0</v>
+      </c>
+      <c r="L30" s="3">
+        <v>0</v>
+      </c>
+      <c r="M30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N30" s="3">
+        <v>0</v>
+      </c>
+      <c r="O30" s="3">
+        <v>5</v>
+      </c>
+      <c r="P30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q30" s="3">
         <v>2</v>
       </c>
-      <c r="L30" s="3">
+      <c r="R30" s="3">
+        <v>0</v>
+      </c>
+      <c r="S30" s="3">
+        <v>1</v>
+      </c>
+      <c r="T30" s="3">
         <v>2</v>
       </c>
-      <c r="M30" s="3">
-        <v>6</v>
-      </c>
-      <c r="N30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P30" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="3">
-        <v>0</v>
-      </c>
-      <c r="R30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="S30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T30" s="3">
-        <v>0</v>
-      </c>
-      <c r="U30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="V30" s="3" t="s">
-        <v>19</v>
+      <c r="U30" s="3">
+        <v>3</v>
+      </c>
+      <c r="V30" s="3">
+        <v>0</v>
       </c>
       <c r="W30" s="3">
         <v>1</v>
       </c>
-      <c r="X30" s="3" t="s">
-        <v>19</v>
+      <c r="X30" s="3">
+        <v>1</v>
       </c>
       <c r="Y30" s="3">
-        <v>4</v>
-      </c>
-      <c r="Z30" s="3" t="s">
-        <v>19</v>
+        <v>2</v>
+      </c>
+      <c r="Z30" s="3">
+        <v>0</v>
       </c>
       <c r="AA30" s="3">
-        <v>1</v>
-      </c>
-      <c r="AB30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AC30" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="AB30" s="3">
+        <v>2</v>
+      </c>
+      <c r="AC30" s="3">
+        <v>1</v>
       </c>
       <c r="AD30" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG30" s="3">
         <v>2</v>
       </c>
-      <c r="AF30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AH30" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI30" s="3"/>
+      <c r="AH30" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI30" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ30" s="3"/>
       <c r="AK30" s="3"/>
       <c r="AL30" s="3"/>
@@ -8501,34 +8549,34 @@
     </row>
     <row r="31" spans="2:61" ht="14.1" customHeight="1">
       <c r="B31" s="14" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="C31" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I31:BI31)</f>
         <v>23</v>
       </c>
       <c r="D31" s="11">
-        <f t="shared" si="14"/>
-        <v>13</v>
+        <f>SUM(I31:V31)</f>
+        <v>11</v>
       </c>
       <c r="E31" s="11">
-        <f t="shared" si="15"/>
-        <v>10</v>
+        <f>SUM(W31:AI31)</f>
+        <v>12</v>
       </c>
       <c r="F31" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ31:AV31)</f>
         <v>0</v>
       </c>
       <c r="G31" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW31:BI31)</f>
         <v>0</v>
       </c>
       <c r="H31" s="11">
-        <f t="shared" si="18"/>
-        <v>24</v>
+        <f>COUNT(I31:BI31)</f>
+        <v>26</v>
       </c>
       <c r="I31" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J31" s="3">
         <v>0</v>
@@ -8537,55 +8585,55 @@
         <v>0</v>
       </c>
       <c r="L31" s="3">
-        <v>0</v>
-      </c>
-      <c r="M31" s="3" t="s">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="M31" s="3">
+        <v>0</v>
       </c>
       <c r="N31" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O31" s="3">
-        <v>5</v>
-      </c>
-      <c r="P31" s="3" t="s">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="P31" s="3">
+        <v>0</v>
       </c>
       <c r="Q31" s="3">
+        <v>0</v>
+      </c>
+      <c r="R31" s="3">
+        <v>1</v>
+      </c>
+      <c r="S31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T31" s="3">
+        <v>1</v>
+      </c>
+      <c r="U31" s="3">
+        <v>1</v>
+      </c>
+      <c r="V31" s="3">
         <v>2</v>
       </c>
-      <c r="R31" s="3">
-        <v>0</v>
-      </c>
-      <c r="S31" s="3">
-        <v>1</v>
-      </c>
-      <c r="T31" s="3">
+      <c r="W31" s="3">
+        <v>0</v>
+      </c>
+      <c r="X31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="3">
         <v>2</v>
       </c>
-      <c r="U31" s="3">
-        <v>3</v>
-      </c>
-      <c r="V31" s="3">
-        <v>0</v>
-      </c>
-      <c r="W31" s="3">
-        <v>1</v>
-      </c>
-      <c r="X31" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y31" s="3">
-        <v>2</v>
-      </c>
-      <c r="Z31" s="3">
-        <v>0</v>
-      </c>
       <c r="AA31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB31" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC31" s="3">
         <v>1</v>
@@ -8597,15 +8645,17 @@
         <v>0</v>
       </c>
       <c r="AF31" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG31" s="3">
         <v>2</v>
       </c>
       <c r="AH31" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI31" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="AI31" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ31" s="3"/>
       <c r="AK31" s="3"/>
       <c r="AL31" s="3"/>
@@ -8638,28 +8688,28 @@
         <v>15</v>
       </c>
       <c r="C32" s="6">
-        <f t="shared" si="13"/>
-        <v>17</v>
+        <f>SUM(I32:BI32)</f>
+        <v>19</v>
       </c>
       <c r="D32" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I32:V32)</f>
         <v>8</v>
       </c>
       <c r="E32" s="11">
-        <f t="shared" si="15"/>
-        <v>9</v>
+        <f>SUM(W32:AI32)</f>
+        <v>11</v>
       </c>
       <c r="F32" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ32:AV32)</f>
         <v>0</v>
       </c>
       <c r="G32" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW32:BI32)</f>
         <v>0</v>
       </c>
       <c r="H32" s="11">
-        <f t="shared" si="18"/>
-        <v>13</v>
+        <f>COUNT(I32:BI32)</f>
+        <v>14</v>
       </c>
       <c r="I32" s="3" t="s">
         <v>19</v>
@@ -8739,7 +8789,9 @@
       <c r="AH32" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AI32" s="3"/>
+      <c r="AI32" s="3">
+        <v>2</v>
+      </c>
       <c r="AJ32" s="3"/>
       <c r="AK32" s="3"/>
       <c r="AL32" s="3"/>
@@ -8772,27 +8824,27 @@
         <v>7</v>
       </c>
       <c r="C33" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I33:BI33)</f>
         <v>16</v>
       </c>
       <c r="D33" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I33:V33)</f>
         <v>10</v>
       </c>
       <c r="E33" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W33:AI33)</f>
         <v>6</v>
       </c>
       <c r="F33" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ33:AV33)</f>
         <v>0</v>
       </c>
       <c r="G33" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW33:BI33)</f>
         <v>0</v>
       </c>
       <c r="H33" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I33:BI33)</f>
         <v>19</v>
       </c>
       <c r="I33" s="3">
@@ -8873,7 +8925,9 @@
       <c r="AH33" s="3">
         <v>0</v>
       </c>
-      <c r="AI33" s="3"/>
+      <c r="AI33" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ33" s="3"/>
       <c r="AK33" s="3"/>
       <c r="AL33" s="3"/>
@@ -8903,73 +8957,73 @@
     </row>
     <row r="34" spans="2:61" ht="14.1" customHeight="1">
       <c r="B34" s="14" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="C34" s="6">
-        <f t="shared" si="13"/>
-        <v>23</v>
+        <f>SUM(I34:BI34)</f>
+        <v>7</v>
       </c>
       <c r="D34" s="11">
-        <f t="shared" si="14"/>
-        <v>11</v>
+        <f>SUM(I34:V34)</f>
+        <v>4</v>
       </c>
       <c r="E34" s="11">
-        <f t="shared" si="15"/>
-        <v>12</v>
+        <f>SUM(W34:AI34)</f>
+        <v>3</v>
       </c>
       <c r="F34" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ34:AV34)</f>
         <v>0</v>
       </c>
       <c r="G34" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW34:BI34)</f>
         <v>0</v>
       </c>
       <c r="H34" s="11">
-        <f t="shared" si="18"/>
-        <v>25</v>
+        <f>COUNT(I34:BI34)</f>
+        <v>16</v>
       </c>
       <c r="I34" s="3">
+        <v>0</v>
+      </c>
+      <c r="J34" s="3">
+        <v>0</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L34" s="3">
+        <v>0</v>
+      </c>
+      <c r="M34" s="3">
+        <v>0</v>
+      </c>
+      <c r="N34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O34" s="3">
+        <v>1</v>
+      </c>
+      <c r="P34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q34" s="3">
+        <v>1</v>
+      </c>
+      <c r="R34" s="3">
+        <v>0</v>
+      </c>
+      <c r="S34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="U34" s="3">
         <v>2</v>
       </c>
-      <c r="J34" s="3">
-        <v>0</v>
-      </c>
-      <c r="K34" s="3">
-        <v>0</v>
-      </c>
-      <c r="L34" s="3">
-        <v>1</v>
-      </c>
-      <c r="M34" s="3">
-        <v>0</v>
-      </c>
-      <c r="N34" s="3">
-        <v>2</v>
-      </c>
-      <c r="O34" s="3">
-        <v>1</v>
-      </c>
-      <c r="P34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="3">
-        <v>0</v>
-      </c>
-      <c r="R34" s="3">
-        <v>1</v>
-      </c>
-      <c r="S34" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T34" s="3">
-        <v>1</v>
-      </c>
-      <c r="U34" s="3">
-        <v>1</v>
-      </c>
-      <c r="V34" s="3">
-        <v>2</v>
+      <c r="V34" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="W34" s="3">
         <v>0</v>
@@ -8978,10 +9032,10 @@
         <v>0</v>
       </c>
       <c r="Y34" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z34" s="3">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="Z34" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AA34" s="3">
         <v>1</v>
@@ -8993,21 +9047,23 @@
         <v>1</v>
       </c>
       <c r="AD34" s="3">
-        <v>1</v>
-      </c>
-      <c r="AE34" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="AE34" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AF34" s="3">
-        <v>3</v>
-      </c>
-      <c r="AG34" s="3">
-        <v>2</v>
-      </c>
-      <c r="AH34" s="3">
-        <v>2</v>
-      </c>
-      <c r="AI34" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="AG34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AH34" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI34" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ34" s="3"/>
       <c r="AK34" s="3"/>
       <c r="AL34" s="3"/>
@@ -9037,40 +9093,40 @@
     </row>
     <row r="35" spans="2:61" ht="14.1" customHeight="1">
       <c r="B35" s="14" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="C35" s="6">
-        <f t="shared" si="13"/>
-        <v>7</v>
+        <f>SUM(I35:BI35)</f>
+        <v>5</v>
       </c>
       <c r="D35" s="11">
-        <f t="shared" si="14"/>
-        <v>4</v>
+        <f>SUM(I35:V35)</f>
+        <v>3</v>
       </c>
       <c r="E35" s="11">
-        <f t="shared" si="15"/>
-        <v>3</v>
+        <f>SUM(W35:AI35)</f>
+        <v>2</v>
       </c>
       <c r="F35" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ35:AV35)</f>
         <v>0</v>
       </c>
       <c r="G35" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW35:BI35)</f>
         <v>0</v>
       </c>
       <c r="H35" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I35:BI35)</f>
         <v>16</v>
       </c>
-      <c r="I35" s="3">
-        <v>0</v>
+      <c r="I35" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="J35" s="3">
         <v>0</v>
       </c>
-      <c r="K35" s="3" t="s">
-        <v>19</v>
+      <c r="K35" s="3">
+        <v>0</v>
       </c>
       <c r="L35" s="3">
         <v>0</v>
@@ -9078,56 +9134,56 @@
       <c r="M35" s="3">
         <v>0</v>
       </c>
-      <c r="N35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O35" s="3">
-        <v>1</v>
-      </c>
-      <c r="P35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q35" s="3">
-        <v>1</v>
-      </c>
-      <c r="R35" s="3">
-        <v>0</v>
-      </c>
-      <c r="S35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T35" s="3" t="s">
-        <v>19</v>
+      <c r="N35" s="3">
+        <v>0</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P35" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="S35" s="3">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3">
+        <v>1</v>
       </c>
       <c r="U35" s="3">
-        <v>2</v>
-      </c>
-      <c r="V35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="W35" s="3">
-        <v>0</v>
-      </c>
-      <c r="X35" s="3">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="V35" s="3">
+        <v>1</v>
+      </c>
+      <c r="W35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="X35" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Y35" s="3">
-        <v>1</v>
-      </c>
-      <c r="Z35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AA35" s="3">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="Z35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AB35" s="3">
         <v>0</v>
       </c>
-      <c r="AC35" s="3">
-        <v>1</v>
-      </c>
-      <c r="AD35" s="3">
-        <v>0</v>
+      <c r="AC35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD35" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AE35" s="3" t="s">
         <v>19</v>
@@ -9135,13 +9191,15 @@
       <c r="AF35" s="3">
         <v>0</v>
       </c>
-      <c r="AG35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AH35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI35" s="3"/>
+      <c r="AG35" s="3">
+        <v>1</v>
+      </c>
+      <c r="AH35" s="3">
+        <v>1</v>
+      </c>
+      <c r="AI35" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ35" s="3"/>
       <c r="AK35" s="3"/>
       <c r="AL35" s="3"/>
@@ -9171,55 +9229,55 @@
     </row>
     <row r="36" spans="2:61" ht="14.1" customHeight="1">
       <c r="B36" s="14" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="C36" s="6">
-        <f t="shared" si="13"/>
-        <v>5</v>
+        <f>SUM(I36:BI36)</f>
+        <v>3</v>
       </c>
       <c r="D36" s="11">
-        <f t="shared" si="14"/>
-        <v>3</v>
+        <f>SUM(I36:V36)</f>
+        <v>0</v>
       </c>
       <c r="E36" s="11">
-        <f t="shared" si="15"/>
-        <v>2</v>
+        <f>SUM(W36:AI36)</f>
+        <v>3</v>
       </c>
       <c r="F36" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ36:AV36)</f>
         <v>0</v>
       </c>
       <c r="G36" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW36:BI36)</f>
         <v>0</v>
       </c>
       <c r="H36" s="11">
-        <f t="shared" si="18"/>
-        <v>16</v>
+        <f>COUNT(I36:BI36)</f>
+        <v>4</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J36" s="3">
-        <v>0</v>
-      </c>
-      <c r="K36" s="3">
-        <v>0</v>
-      </c>
-      <c r="L36" s="3">
-        <v>0</v>
-      </c>
-      <c r="M36" s="3">
-        <v>0</v>
-      </c>
-      <c r="N36" s="3">
-        <v>0</v>
+      <c r="J36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="O36" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="P36" s="3">
-        <v>0</v>
+      <c r="P36" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Q36" s="3" t="s">
         <v>19</v>
@@ -9227,17 +9285,17 @@
       <c r="R36" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="S36" s="3">
-        <v>0</v>
-      </c>
-      <c r="T36" s="3">
-        <v>1</v>
-      </c>
-      <c r="U36" s="3">
-        <v>1</v>
-      </c>
-      <c r="V36" s="3">
-        <v>1</v>
+      <c r="S36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="U36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="V36" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="W36" s="3" t="s">
         <v>19</v>
@@ -9245,11 +9303,11 @@
       <c r="X36" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Y36" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z36" s="3">
-        <v>0</v>
+      <c r="Y36" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z36" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AA36" s="3" t="s">
         <v>19</v>
@@ -9266,8 +9324,8 @@
       <c r="AE36" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AF36" s="3">
-        <v>0</v>
+      <c r="AF36" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AG36" s="3">
         <v>1</v>
@@ -9275,7 +9333,9 @@
       <c r="AH36" s="3">
         <v>1</v>
       </c>
-      <c r="AI36" s="3"/>
+      <c r="AI36" s="3">
+        <v>1</v>
+      </c>
       <c r="AJ36" s="3"/>
       <c r="AK36" s="3"/>
       <c r="AL36" s="3"/>
@@ -9308,27 +9368,27 @@
         <v>10</v>
       </c>
       <c r="C37" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I37:BI37)</f>
         <v>0</v>
       </c>
       <c r="D37" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I37:V37)</f>
         <v>0</v>
       </c>
       <c r="E37" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W37:AI37)</f>
         <v>0</v>
       </c>
       <c r="F37" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ37:AV37)</f>
         <v>0</v>
       </c>
       <c r="G37" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW37:BI37)</f>
         <v>0</v>
       </c>
       <c r="H37" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I37:BI37)</f>
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
@@ -9409,7 +9469,9 @@
       <c r="AH37" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AI37" s="3"/>
+      <c r="AI37" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AJ37" s="3"/>
       <c r="AK37" s="3"/>
       <c r="AL37" s="3"/>
@@ -9438,414 +9500,416 @@
       <c r="BI37" s="3"/>
     </row>
     <row r="38" spans="2:61" ht="14.1" customHeight="1">
-      <c r="B38" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C38" s="6">
-        <f t="shared" si="13"/>
-        <v>2</v>
-      </c>
-      <c r="D38" s="11">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="E38" s="11">
-        <f t="shared" si="15"/>
-        <v>2</v>
-      </c>
-      <c r="F38" s="11">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="G38" s="11">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="H38" s="11">
-        <f t="shared" si="18"/>
-        <v>3</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="R38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="S38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="U38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="V38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="W38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="X38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Y38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AA38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB38" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AD38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AF38" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AG38" s="3">
-        <v>1</v>
-      </c>
-      <c r="AH38" s="3">
-        <v>1</v>
-      </c>
-      <c r="AI38" s="3"/>
-      <c r="AJ38" s="3"/>
-      <c r="AK38" s="3"/>
-      <c r="AL38" s="3"/>
-      <c r="AM38" s="3"/>
-      <c r="AN38" s="3"/>
-      <c r="AO38" s="3"/>
-      <c r="AP38" s="3"/>
-      <c r="AQ38" s="3"/>
-      <c r="AR38" s="3"/>
-      <c r="AS38" s="3"/>
-      <c r="AT38" s="3"/>
-      <c r="AU38" s="3"/>
-      <c r="AV38" s="3"/>
-      <c r="AW38" s="3"/>
-      <c r="AX38" s="3"/>
-      <c r="AY38" s="3"/>
-      <c r="AZ38" s="3"/>
-      <c r="BA38" s="3"/>
-      <c r="BB38" s="3"/>
-      <c r="BC38" s="3"/>
-      <c r="BD38" s="3"/>
-      <c r="BE38" s="3"/>
-      <c r="BF38" s="3"/>
-      <c r="BG38" s="3"/>
-      <c r="BH38" s="3"/>
-      <c r="BI38" s="3"/>
+      <c r="B38" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I38" s="5">
+        <v>46025</v>
+      </c>
+      <c r="J38" s="5">
+        <f>I38+7</f>
+        <v>46032</v>
+      </c>
+      <c r="K38" s="5">
+        <f t="shared" ref="K38:BH38" si="7">J38+7</f>
+        <v>46039</v>
+      </c>
+      <c r="L38" s="5">
+        <f t="shared" si="7"/>
+        <v>46046</v>
+      </c>
+      <c r="M38" s="5">
+        <f t="shared" si="7"/>
+        <v>46053</v>
+      </c>
+      <c r="N38" s="5">
+        <f t="shared" si="7"/>
+        <v>46060</v>
+      </c>
+      <c r="O38" s="5">
+        <f t="shared" si="7"/>
+        <v>46067</v>
+      </c>
+      <c r="P38" s="5">
+        <v>46070</v>
+      </c>
+      <c r="Q38" s="5">
+        <f>O38+7</f>
+        <v>46074</v>
+      </c>
+      <c r="R38" s="5">
+        <f t="shared" si="7"/>
+        <v>46081</v>
+      </c>
+      <c r="S38" s="5">
+        <f t="shared" si="7"/>
+        <v>46088</v>
+      </c>
+      <c r="T38" s="5">
+        <f t="shared" si="7"/>
+        <v>46095</v>
+      </c>
+      <c r="U38" s="5">
+        <f t="shared" si="7"/>
+        <v>46102</v>
+      </c>
+      <c r="V38" s="5">
+        <f t="shared" si="7"/>
+        <v>46109</v>
+      </c>
+      <c r="W38" s="5">
+        <f t="shared" si="7"/>
+        <v>46116</v>
+      </c>
+      <c r="X38" s="5">
+        <f t="shared" si="7"/>
+        <v>46123</v>
+      </c>
+      <c r="Y38" s="5">
+        <f t="shared" si="7"/>
+        <v>46130</v>
+      </c>
+      <c r="Z38" s="5">
+        <f t="shared" si="7"/>
+        <v>46137</v>
+      </c>
+      <c r="AA38" s="5">
+        <f t="shared" si="7"/>
+        <v>46144</v>
+      </c>
+      <c r="AB38" s="5">
+        <f t="shared" si="7"/>
+        <v>46151</v>
+      </c>
+      <c r="AC38" s="5">
+        <f t="shared" si="7"/>
+        <v>46158</v>
+      </c>
+      <c r="AD38" s="5">
+        <f t="shared" si="7"/>
+        <v>46165</v>
+      </c>
+      <c r="AE38" s="5">
+        <f t="shared" si="7"/>
+        <v>46172</v>
+      </c>
+      <c r="AF38" s="5">
+        <f t="shared" si="7"/>
+        <v>46179</v>
+      </c>
+      <c r="AG38" s="5">
+        <f t="shared" si="7"/>
+        <v>46186</v>
+      </c>
+      <c r="AH38" s="5">
+        <f t="shared" si="7"/>
+        <v>46193</v>
+      </c>
+      <c r="AI38" s="5">
+        <f t="shared" si="7"/>
+        <v>46200</v>
+      </c>
+      <c r="AJ38" s="5">
+        <f t="shared" si="7"/>
+        <v>46207</v>
+      </c>
+      <c r="AK38" s="5">
+        <f t="shared" si="7"/>
+        <v>46214</v>
+      </c>
+      <c r="AL38" s="5">
+        <f t="shared" si="7"/>
+        <v>46221</v>
+      </c>
+      <c r="AM38" s="5">
+        <f t="shared" si="7"/>
+        <v>46228</v>
+      </c>
+      <c r="AN38" s="5">
+        <f t="shared" si="7"/>
+        <v>46235</v>
+      </c>
+      <c r="AO38" s="5">
+        <f t="shared" si="7"/>
+        <v>46242</v>
+      </c>
+      <c r="AP38" s="5">
+        <f t="shared" si="7"/>
+        <v>46249</v>
+      </c>
+      <c r="AQ38" s="5">
+        <f t="shared" si="7"/>
+        <v>46256</v>
+      </c>
+      <c r="AR38" s="5">
+        <f t="shared" si="7"/>
+        <v>46263</v>
+      </c>
+      <c r="AS38" s="5">
+        <f t="shared" si="7"/>
+        <v>46270</v>
+      </c>
+      <c r="AT38" s="5">
+        <f t="shared" si="7"/>
+        <v>46277</v>
+      </c>
+      <c r="AU38" s="5">
+        <f t="shared" si="7"/>
+        <v>46284</v>
+      </c>
+      <c r="AV38" s="5">
+        <f t="shared" si="7"/>
+        <v>46291</v>
+      </c>
+      <c r="AW38" s="5">
+        <f t="shared" si="7"/>
+        <v>46298</v>
+      </c>
+      <c r="AX38" s="5">
+        <f t="shared" si="7"/>
+        <v>46305</v>
+      </c>
+      <c r="AY38" s="5">
+        <f t="shared" si="7"/>
+        <v>46312</v>
+      </c>
+      <c r="AZ38" s="5">
+        <f t="shared" si="7"/>
+        <v>46319</v>
+      </c>
+      <c r="BA38" s="5">
+        <f t="shared" si="7"/>
+        <v>46326</v>
+      </c>
+      <c r="BB38" s="5">
+        <f t="shared" si="7"/>
+        <v>46333</v>
+      </c>
+      <c r="BC38" s="5">
+        <f t="shared" si="7"/>
+        <v>46340</v>
+      </c>
+      <c r="BD38" s="5">
+        <f t="shared" si="7"/>
+        <v>46347</v>
+      </c>
+      <c r="BE38" s="5">
+        <f t="shared" si="7"/>
+        <v>46354</v>
+      </c>
+      <c r="BF38" s="5">
+        <f t="shared" si="7"/>
+        <v>46361</v>
+      </c>
+      <c r="BG38" s="5">
+        <f t="shared" si="7"/>
+        <v>46368</v>
+      </c>
+      <c r="BH38" s="5">
+        <f t="shared" si="7"/>
+        <v>46375</v>
+      </c>
+      <c r="BI38" s="5">
+        <f t="shared" ref="BI38" si="8">BH38+7</f>
+        <v>46382</v>
+      </c>
     </row>
     <row r="39" spans="2:61" ht="14.1" customHeight="1">
-      <c r="B39" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I39" s="5">
-        <v>46025</v>
-      </c>
-      <c r="J39" s="5">
-        <f>I39+7</f>
-        <v>46032</v>
-      </c>
-      <c r="K39" s="5">
-        <f t="shared" ref="K39:BH39" si="19">J39+7</f>
-        <v>46039</v>
-      </c>
-      <c r="L39" s="5">
-        <f t="shared" si="19"/>
-        <v>46046</v>
-      </c>
-      <c r="M39" s="5">
-        <f t="shared" si="19"/>
-        <v>46053</v>
-      </c>
-      <c r="N39" s="5">
-        <f t="shared" si="19"/>
-        <v>46060</v>
-      </c>
-      <c r="O39" s="5">
-        <f t="shared" si="19"/>
-        <v>46067</v>
-      </c>
-      <c r="P39" s="5">
-        <v>46070</v>
-      </c>
-      <c r="Q39" s="5">
-        <f>O39+7</f>
-        <v>46074</v>
-      </c>
-      <c r="R39" s="5">
-        <f t="shared" si="19"/>
-        <v>46081</v>
-      </c>
-      <c r="S39" s="5">
-        <f t="shared" si="19"/>
-        <v>46088</v>
-      </c>
-      <c r="T39" s="5">
-        <f t="shared" si="19"/>
-        <v>46095</v>
-      </c>
-      <c r="U39" s="5">
-        <f t="shared" si="19"/>
-        <v>46102</v>
-      </c>
-      <c r="V39" s="5">
-        <f t="shared" si="19"/>
-        <v>46109</v>
-      </c>
-      <c r="W39" s="5">
-        <f t="shared" si="19"/>
-        <v>46116</v>
-      </c>
-      <c r="X39" s="5">
-        <f t="shared" si="19"/>
-        <v>46123</v>
-      </c>
-      <c r="Y39" s="5">
-        <f t="shared" si="19"/>
-        <v>46130</v>
-      </c>
-      <c r="Z39" s="5">
-        <f t="shared" si="19"/>
-        <v>46137</v>
-      </c>
-      <c r="AA39" s="5">
-        <f t="shared" si="19"/>
-        <v>46144</v>
-      </c>
-      <c r="AB39" s="5">
-        <f t="shared" si="19"/>
-        <v>46151</v>
-      </c>
-      <c r="AC39" s="5">
-        <f t="shared" si="19"/>
-        <v>46158</v>
-      </c>
-      <c r="AD39" s="5">
-        <f t="shared" si="19"/>
-        <v>46165</v>
-      </c>
-      <c r="AE39" s="5">
-        <f t="shared" si="19"/>
-        <v>46172</v>
-      </c>
-      <c r="AF39" s="5">
-        <f t="shared" si="19"/>
-        <v>46179</v>
-      </c>
-      <c r="AG39" s="5">
-        <f t="shared" si="19"/>
-        <v>46186</v>
-      </c>
-      <c r="AH39" s="5">
-        <f t="shared" si="19"/>
-        <v>46193</v>
-      </c>
-      <c r="AI39" s="5">
-        <f t="shared" si="19"/>
-        <v>46200</v>
-      </c>
-      <c r="AJ39" s="5">
-        <f t="shared" si="19"/>
-        <v>46207</v>
-      </c>
-      <c r="AK39" s="5">
-        <f t="shared" si="19"/>
-        <v>46214</v>
-      </c>
-      <c r="AL39" s="5">
-        <f t="shared" si="19"/>
-        <v>46221</v>
-      </c>
-      <c r="AM39" s="5">
-        <f t="shared" si="19"/>
-        <v>46228</v>
-      </c>
-      <c r="AN39" s="5">
-        <f t="shared" si="19"/>
-        <v>46235</v>
-      </c>
-      <c r="AO39" s="5">
-        <f t="shared" si="19"/>
-        <v>46242</v>
-      </c>
-      <c r="AP39" s="5">
-        <f t="shared" si="19"/>
-        <v>46249</v>
-      </c>
-      <c r="AQ39" s="5">
-        <f t="shared" si="19"/>
-        <v>46256</v>
-      </c>
-      <c r="AR39" s="5">
-        <f t="shared" si="19"/>
-        <v>46263</v>
-      </c>
-      <c r="AS39" s="5">
-        <f t="shared" si="19"/>
-        <v>46270</v>
-      </c>
-      <c r="AT39" s="5">
-        <f t="shared" si="19"/>
-        <v>46277</v>
-      </c>
-      <c r="AU39" s="5">
-        <f t="shared" si="19"/>
-        <v>46284</v>
-      </c>
-      <c r="AV39" s="5">
-        <f t="shared" si="19"/>
-        <v>46291</v>
-      </c>
-      <c r="AW39" s="5">
-        <f t="shared" si="19"/>
-        <v>46298</v>
-      </c>
-      <c r="AX39" s="5">
-        <f t="shared" si="19"/>
-        <v>46305</v>
-      </c>
-      <c r="AY39" s="5">
-        <f t="shared" si="19"/>
-        <v>46312</v>
-      </c>
-      <c r="AZ39" s="5">
-        <f t="shared" si="19"/>
-        <v>46319</v>
-      </c>
-      <c r="BA39" s="5">
-        <f t="shared" si="19"/>
-        <v>46326</v>
-      </c>
-      <c r="BB39" s="5">
-        <f t="shared" si="19"/>
-        <v>46333</v>
-      </c>
-      <c r="BC39" s="5">
-        <f t="shared" si="19"/>
-        <v>46340</v>
-      </c>
-      <c r="BD39" s="5">
-        <f t="shared" si="19"/>
-        <v>46347</v>
-      </c>
-      <c r="BE39" s="5">
-        <f t="shared" si="19"/>
-        <v>46354</v>
-      </c>
-      <c r="BF39" s="5">
-        <f t="shared" si="19"/>
-        <v>46361</v>
-      </c>
-      <c r="BG39" s="5">
-        <f t="shared" si="19"/>
-        <v>46368</v>
-      </c>
-      <c r="BH39" s="5">
-        <f t="shared" si="19"/>
-        <v>46375</v>
-      </c>
-      <c r="BI39" s="5">
-        <f t="shared" ref="BI39" si="20">BH39+7</f>
-        <v>46382</v>
-      </c>
+      <c r="B39" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="6">
+        <f>SUM(I39:BI39)</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="11">
+        <f t="shared" ref="D39:D40" si="9">SUM(I39:V39)</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="11">
+        <f t="shared" ref="E39:E40" si="10">SUM(W39:AI39)</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="11">
+        <f t="shared" ref="F39:F40" si="11">SUM(AJ39:AV39)</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="11">
+        <f t="shared" ref="G39:G40" si="12">SUM(AW39:BI39)</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="11">
+        <f t="shared" ref="H39:H40" si="13">COUNT(I39:BI39)</f>
+        <v>22</v>
+      </c>
+      <c r="I39" s="3">
+        <v>0</v>
+      </c>
+      <c r="J39" s="3">
+        <v>0</v>
+      </c>
+      <c r="K39" s="3">
+        <v>0</v>
+      </c>
+      <c r="L39" s="3">
+        <v>0</v>
+      </c>
+      <c r="M39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N39" s="3">
+        <v>0</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q39" s="3">
+        <v>0</v>
+      </c>
+      <c r="R39" s="3">
+        <v>0</v>
+      </c>
+      <c r="S39" s="3">
+        <v>0</v>
+      </c>
+      <c r="T39" s="3">
+        <v>0</v>
+      </c>
+      <c r="U39" s="3">
+        <v>0</v>
+      </c>
+      <c r="V39" s="3">
+        <v>0</v>
+      </c>
+      <c r="W39" s="3">
+        <v>0</v>
+      </c>
+      <c r="X39" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI39" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ39" s="3"/>
+      <c r="AK39" s="3"/>
+      <c r="AL39" s="3"/>
+      <c r="AM39" s="3"/>
+      <c r="AN39" s="3"/>
+      <c r="AO39" s="3"/>
+      <c r="AP39" s="3"/>
+      <c r="AQ39" s="3"/>
+      <c r="AR39" s="3"/>
+      <c r="AS39" s="3"/>
+      <c r="AT39" s="3"/>
+      <c r="AU39" s="3"/>
+      <c r="AV39" s="3"/>
+      <c r="AW39" s="3"/>
+      <c r="AX39" s="3"/>
+      <c r="AY39" s="3"/>
+      <c r="AZ39" s="3"/>
+      <c r="BA39" s="3"/>
+      <c r="BB39" s="3"/>
+      <c r="BC39" s="3"/>
+      <c r="BD39" s="3"/>
+      <c r="BE39" s="3"/>
+      <c r="BF39" s="3"/>
+      <c r="BG39" s="3"/>
+      <c r="BH39" s="3"/>
+      <c r="BI39" s="3"/>
     </row>
     <row r="40" spans="2:61" ht="14.1" customHeight="1">
       <c r="B40" s="14" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C40" s="6">
         <f>SUM(I40:BI40)</f>
         <v>0</v>
       </c>
       <c r="D40" s="11">
-        <f t="shared" ref="D40:D41" si="21">SUM(I40:V40)</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="E40" s="11">
-        <f t="shared" ref="E40:E41" si="22">SUM(W40:AI40)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F40" s="11">
-        <f t="shared" ref="F40:F41" si="23">SUM(AJ40:AV40)</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="G40" s="11">
-        <f t="shared" ref="G40:G41" si="24">SUM(AW40:BI40)</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="H40" s="11">
-        <f t="shared" ref="H40:H41" si="25">COUNT(I40:BI40)</f>
-        <v>21</v>
-      </c>
-      <c r="I40" s="3">
-        <v>0</v>
+        <f t="shared" si="13"/>
+        <v>20</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="J40" s="3">
         <v>0</v>
       </c>
-      <c r="K40" s="3">
-        <v>0</v>
-      </c>
-      <c r="L40" s="3">
-        <v>0</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>19</v>
+      <c r="K40" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M40" s="3">
+        <v>0</v>
       </c>
       <c r="N40" s="3">
         <v>0</v>
@@ -9883,14 +9947,14 @@
       <c r="Y40" s="3">
         <v>0</v>
       </c>
-      <c r="Z40" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA40" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB40" s="3">
-        <v>0</v>
+      <c r="Z40" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AC40" s="3">
         <v>0</v>
@@ -9907,10 +9971,12 @@
       <c r="AG40" s="3">
         <v>0</v>
       </c>
-      <c r="AH40" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI40" s="3"/>
+      <c r="AH40" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI40" s="3">
+        <v>0</v>
+      </c>
       <c r="AJ40" s="3"/>
       <c r="AK40" s="3"/>
       <c r="AL40" s="3"/>
@@ -9938,140 +10004,6 @@
       <c r="BH40" s="3"/>
       <c r="BI40" s="3"/>
     </row>
-    <row r="41" spans="2:61" ht="14.1" customHeight="1">
-      <c r="B41" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C41" s="6">
-        <f>SUM(I41:BI41)</f>
-        <v>0</v>
-      </c>
-      <c r="D41" s="11">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="E41" s="11">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
-      <c r="F41" s="11">
-        <f t="shared" si="23"/>
-        <v>0</v>
-      </c>
-      <c r="G41" s="11">
-        <f t="shared" si="24"/>
-        <v>0</v>
-      </c>
-      <c r="H41" s="11">
-        <f t="shared" si="25"/>
-        <v>19</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J41" s="3">
-        <v>0</v>
-      </c>
-      <c r="K41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M41" s="3">
-        <v>0</v>
-      </c>
-      <c r="N41" s="3">
-        <v>0</v>
-      </c>
-      <c r="O41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q41" s="3">
-        <v>0</v>
-      </c>
-      <c r="R41" s="3">
-        <v>0</v>
-      </c>
-      <c r="S41" s="3">
-        <v>0</v>
-      </c>
-      <c r="T41" s="3">
-        <v>0</v>
-      </c>
-      <c r="U41" s="3">
-        <v>0</v>
-      </c>
-      <c r="V41" s="3">
-        <v>0</v>
-      </c>
-      <c r="W41" s="3">
-        <v>0</v>
-      </c>
-      <c r="X41" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y41" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AA41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB41" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AC41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH41" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI41" s="3"/>
-      <c r="AJ41" s="3"/>
-      <c r="AK41" s="3"/>
-      <c r="AL41" s="3"/>
-      <c r="AM41" s="3"/>
-      <c r="AN41" s="3"/>
-      <c r="AO41" s="3"/>
-      <c r="AP41" s="3"/>
-      <c r="AQ41" s="3"/>
-      <c r="AR41" s="3"/>
-      <c r="AS41" s="3"/>
-      <c r="AT41" s="3"/>
-      <c r="AU41" s="3"/>
-      <c r="AV41" s="3"/>
-      <c r="AW41" s="3"/>
-      <c r="AX41" s="3"/>
-      <c r="AY41" s="3"/>
-      <c r="AZ41" s="3"/>
-      <c r="BA41" s="3"/>
-      <c r="BB41" s="3"/>
-      <c r="BC41" s="3"/>
-      <c r="BD41" s="3"/>
-      <c r="BE41" s="3"/>
-      <c r="BF41" s="3"/>
-      <c r="BG41" s="3"/>
-      <c r="BH41" s="3"/>
-      <c r="BI41" s="3"/>
-    </row>
   </sheetData>
   <sortState ref="B4:AI17">
     <sortCondition descending="1" ref="C4:C17"/>
@@ -10083,7 +10015,7 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="E18:E20 E39:E41 E31:E34 E7:E9" formulaRange="1"/>
+    <ignoredError sqref="E19:E20 F19:F20 E38:E40 E24:F37 F38:F40 F18 E18 E4:F17" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update player data with new statistics and game records
</commit_message>
<xml_diff>
--- a/Pontuação 2026.xlsx
+++ b/Pontuação 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luan-\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0F8751-E65A-4C0B-B188-230FDED1502F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31369FC3-FDBA-4ECA-9A02-D347394C7034}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="41">
   <si>
     <t>Atletas</t>
   </si>
@@ -4570,16 +4570,15 @@
     <col min="23" max="23" width="5.5703125" style="1" hidden="1" customWidth="1"/>
     <col min="24" max="26" width="6.5703125" style="1" hidden="1" customWidth="1"/>
     <col min="27" max="28" width="5.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="6.85546875" style="1" hidden="1" customWidth="1"/>
-    <col min="30" max="31" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="5.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="35" width="6.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="4.5703125" style="1" hidden="1" customWidth="1"/>
-    <col min="37" max="39" width="5.5703125" style="1" hidden="1" customWidth="1"/>
-    <col min="40" max="41" width="6.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="42" max="44" width="7.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="45" max="45" width="5" style="1" hidden="1" customWidth="1"/>
-    <col min="46" max="48" width="6" style="1" hidden="1" customWidth="1"/>
+    <col min="29" max="31" width="6.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="32" max="32" width="5.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="33" max="35" width="6.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="4.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="39" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="41" width="6.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="44" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="48" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="5.28515625" style="1" hidden="1" customWidth="1"/>
     <col min="50" max="53" width="6.28515625" style="1" hidden="1" customWidth="1"/>
     <col min="54" max="54" width="5.85546875" style="1" hidden="1" customWidth="1"/>
@@ -4894,27 +4893,27 @@
         <v>40</v>
       </c>
       <c r="C4" s="6">
-        <f>SUM(I4:BI4)</f>
+        <f t="shared" ref="C4:C17" si="2">SUM(I4:BI4)</f>
         <v>53</v>
       </c>
       <c r="D4" s="11">
-        <f>SUM(I4:V4)</f>
+        <f t="shared" ref="D4:D17" si="3">SUM(I4:V4)</f>
         <v>29</v>
       </c>
       <c r="E4" s="11">
-        <f>SUM(W4:AI4)</f>
+        <f t="shared" ref="E4:E17" si="4">SUM(W4:AI4)</f>
         <v>24</v>
       </c>
       <c r="F4" s="11">
-        <f>SUM(AJ4:AV4)</f>
+        <f t="shared" ref="F4:F17" si="5">SUM(AJ4:AV4)</f>
         <v>0</v>
       </c>
       <c r="G4" s="11">
-        <f>SUM(AW4:BI4)</f>
+        <f t="shared" ref="G4:G17" si="6">SUM(AW4:BI4)</f>
         <v>0</v>
       </c>
       <c r="H4" s="11">
-        <f>COUNT(I4:BI4)</f>
+        <f t="shared" ref="H4:H17" si="7">COUNT(I4:BI4)</f>
         <v>23</v>
       </c>
       <c r="I4" s="3">
@@ -4998,7 +4997,9 @@
       <c r="AI4" s="3">
         <v>3</v>
       </c>
-      <c r="AJ4" s="3"/>
+      <c r="AJ4" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK4" s="3"/>
       <c r="AL4" s="3"/>
       <c r="AM4" s="3"/>
@@ -5030,28 +5031,28 @@
         <v>9</v>
       </c>
       <c r="C5" s="6">
-        <f>SUM(I5:BI5)</f>
+        <f t="shared" si="2"/>
         <v>37</v>
       </c>
       <c r="D5" s="11">
-        <f>SUM(I5:V5)</f>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="E5" s="11">
-        <f>SUM(W5:AI5)</f>
+        <f t="shared" si="4"/>
         <v>21</v>
       </c>
       <c r="F5" s="11">
-        <f>SUM(AJ5:AV5)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G5" s="11">
-        <f>SUM(AW5:BI5)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H5" s="11">
-        <f>COUNT(I5:BI5)</f>
-        <v>23</v>
+        <f t="shared" si="7"/>
+        <v>24</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>19</v>
@@ -5134,7 +5135,9 @@
       <c r="AI5" s="3">
         <v>3</v>
       </c>
-      <c r="AJ5" s="3"/>
+      <c r="AJ5" s="3">
+        <v>0</v>
+      </c>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
       <c r="AM5" s="3"/>
@@ -5166,28 +5169,28 @@
         <v>33</v>
       </c>
       <c r="C6" s="6">
-        <f>SUM(I6:BI6)</f>
-        <v>34</v>
+        <f t="shared" si="2"/>
+        <v>37</v>
       </c>
       <c r="D6" s="11">
-        <f>SUM(I6:V6)</f>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="E6" s="11">
-        <f>SUM(W6:AI6)</f>
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="F6" s="11">
-        <f>SUM(AJ6:AV6)</f>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>3</v>
       </c>
       <c r="G6" s="11">
-        <f>SUM(AW6:BI6)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H6" s="11">
-        <f>COUNT(I6:BI6)</f>
-        <v>22</v>
+        <f t="shared" si="7"/>
+        <v>23</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>19</v>
@@ -5270,7 +5273,9 @@
       <c r="AI6" s="3">
         <v>0</v>
       </c>
-      <c r="AJ6" s="3"/>
+      <c r="AJ6" s="3">
+        <v>3</v>
+      </c>
       <c r="AK6" s="3"/>
       <c r="AL6" s="3"/>
       <c r="AM6" s="3"/>
@@ -5302,28 +5307,28 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <f>SUM(I7:BI7)</f>
+        <f t="shared" si="2"/>
         <v>32</v>
       </c>
       <c r="D7" s="11">
-        <f>SUM(I7:V7)</f>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="E7" s="11">
-        <f>SUM(W7:AI7)</f>
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="F7" s="11">
-        <f>SUM(AJ7:AV7)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G7" s="11">
-        <f>SUM(AW7:BI7)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H7" s="11">
-        <f>COUNT(I7:BI7)</f>
-        <v>26</v>
+        <f t="shared" si="7"/>
+        <v>27</v>
       </c>
       <c r="I7" s="3">
         <v>3</v>
@@ -5406,7 +5411,9 @@
       <c r="AI7" s="3">
         <v>0</v>
       </c>
-      <c r="AJ7" s="3"/>
+      <c r="AJ7" s="3">
+        <v>0</v>
+      </c>
       <c r="AK7" s="3"/>
       <c r="AL7" s="3"/>
       <c r="AM7" s="3"/>
@@ -5438,28 +5445,28 @@
         <v>36</v>
       </c>
       <c r="C8" s="6">
-        <f>SUM(I8:BI8)</f>
+        <f t="shared" si="2"/>
         <v>29</v>
       </c>
       <c r="D8" s="11">
-        <f>SUM(I8:V8)</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="E8" s="11">
-        <f>SUM(W8:AI8)</f>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="F8" s="11">
-        <f>SUM(AJ8:AV8)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G8" s="11">
-        <f>SUM(AW8:BI8)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H8" s="11">
-        <f>COUNT(I8:BI8)</f>
-        <v>17</v>
+        <f t="shared" si="7"/>
+        <v>18</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>19</v>
@@ -5542,7 +5549,9 @@
       <c r="AI8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ8" s="3"/>
+      <c r="AJ8" s="3">
+        <v>0</v>
+      </c>
       <c r="AK8" s="3"/>
       <c r="AL8" s="3"/>
       <c r="AM8" s="3"/>
@@ -5574,28 +5583,28 @@
         <v>18</v>
       </c>
       <c r="C9" s="6">
-        <f>SUM(I9:BI9)</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="D9" s="11">
-        <f>SUM(I9:V9)</f>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="E9" s="11">
-        <f>SUM(W9:AI9)</f>
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="F9" s="11">
-        <f>SUM(AJ9:AV9)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G9" s="11">
-        <f>SUM(AW9:BI9)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H9" s="11">
-        <f>COUNT(I9:BI9)</f>
-        <v>25</v>
+        <f t="shared" si="7"/>
+        <v>26</v>
       </c>
       <c r="I9" s="3">
         <v>3</v>
@@ -5678,7 +5687,9 @@
       <c r="AI9" s="3">
         <v>0</v>
       </c>
-      <c r="AJ9" s="3"/>
+      <c r="AJ9" s="3">
+        <v>0</v>
+      </c>
       <c r="AK9" s="3"/>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
@@ -5710,27 +5721,27 @@
         <v>15</v>
       </c>
       <c r="C10" s="6">
-        <f>SUM(I10:BI10)</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="D10" s="11">
-        <f>SUM(I10:V10)</f>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="E10" s="11">
-        <f>SUM(W10:AI10)</f>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="F10" s="11">
-        <f>SUM(AJ10:AV10)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G10" s="11">
-        <f>SUM(AW10:BI10)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H10" s="11">
-        <f>COUNT(I10:BI10)</f>
+        <f t="shared" si="7"/>
         <v>15</v>
       </c>
       <c r="I10" s="3" t="s">
@@ -5814,7 +5825,9 @@
       <c r="AI10" s="3">
         <v>3</v>
       </c>
-      <c r="AJ10" s="3"/>
+      <c r="AJ10" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK10" s="3"/>
       <c r="AL10" s="3"/>
       <c r="AM10" s="3"/>
@@ -5846,28 +5859,28 @@
         <v>7</v>
       </c>
       <c r="C11" s="6">
-        <f>SUM(I11:BI11)</f>
+        <f t="shared" si="2"/>
         <v>26</v>
       </c>
       <c r="D11" s="11">
-        <f>SUM(I11:V11)</f>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="E11" s="11">
-        <f>SUM(W11:AI11)</f>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="F11" s="11">
-        <f>SUM(AJ11:AV11)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G11" s="11">
-        <f>SUM(AW11:BI11)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H11" s="11">
-        <f>COUNT(I11:BI11)</f>
-        <v>19</v>
+        <f t="shared" si="7"/>
+        <v>20</v>
       </c>
       <c r="I11" s="3">
         <v>3</v>
@@ -5950,7 +5963,9 @@
       <c r="AI11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ11" s="3"/>
+      <c r="AJ11" s="3">
+        <v>0</v>
+      </c>
       <c r="AK11" s="3"/>
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
@@ -5982,29 +5997,29 @@
         <v>5</v>
       </c>
       <c r="C12" s="6">
-        <f>SUM(I12:BI12)</f>
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="D12" s="11">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="E12" s="11">
+        <f t="shared" si="4"/>
+        <v>9</v>
+      </c>
+      <c r="F12" s="11">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="G12" s="11">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="11">
+        <f t="shared" si="7"/>
         <v>25</v>
       </c>
-      <c r="D12" s="11">
-        <f>SUM(I12:V12)</f>
-        <v>16</v>
-      </c>
-      <c r="E12" s="11">
-        <f>SUM(W12:AI12)</f>
-        <v>9</v>
-      </c>
-      <c r="F12" s="11">
-        <f>SUM(AJ12:AV12)</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="11">
-        <f>SUM(AW12:BI12)</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="11">
-        <f>COUNT(I12:BI12)</f>
-        <v>24</v>
-      </c>
       <c r="I12" s="3">
         <v>3</v>
       </c>
@@ -6086,7 +6101,9 @@
       <c r="AI12" s="3">
         <v>0</v>
       </c>
-      <c r="AJ12" s="3"/>
+      <c r="AJ12" s="3">
+        <v>3</v>
+      </c>
       <c r="AK12" s="3"/>
       <c r="AL12" s="3"/>
       <c r="AM12" s="3"/>
@@ -6118,27 +6135,27 @@
         <v>11</v>
       </c>
       <c r="C13" s="6">
-        <f>SUM(I13:BI13)</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="D13" s="11">
-        <f>SUM(I13:V13)</f>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="E13" s="11">
-        <f>SUM(W13:AI13)</f>
+        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="F13" s="11">
-        <f>SUM(AJ13:AV13)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G13" s="11">
-        <f>SUM(AW13:BI13)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H13" s="11">
-        <f>COUNT(I13:BI13)</f>
+        <f t="shared" si="7"/>
         <v>21</v>
       </c>
       <c r="I13" s="3">
@@ -6222,7 +6239,9 @@
       <c r="AI13" s="3">
         <v>0</v>
       </c>
-      <c r="AJ13" s="3"/>
+      <c r="AJ13" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK13" s="3"/>
       <c r="AL13" s="3"/>
       <c r="AM13" s="3"/>
@@ -6254,28 +6273,28 @@
         <v>3</v>
       </c>
       <c r="C14" s="6">
-        <f>SUM(I14:BI14)</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="D14" s="11">
-        <f>SUM(I14:V14)</f>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="E14" s="11">
-        <f>SUM(W14:AI14)</f>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="F14" s="11">
-        <f>SUM(AJ14:AV14)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G14" s="11">
-        <f>SUM(AW14:BI14)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H14" s="11">
-        <f>COUNT(I14:BI14)</f>
-        <v>23</v>
+        <f t="shared" si="7"/>
+        <v>24</v>
       </c>
       <c r="I14" s="3">
         <v>0</v>
@@ -6358,7 +6377,9 @@
       <c r="AI14" s="3">
         <v>0</v>
       </c>
-      <c r="AJ14" s="3"/>
+      <c r="AJ14" s="3">
+        <v>0</v>
+      </c>
       <c r="AK14" s="3"/>
       <c r="AL14" s="3"/>
       <c r="AM14" s="3"/>
@@ -6390,28 +6411,28 @@
         <v>6</v>
       </c>
       <c r="C15" s="6">
-        <f>SUM(I15:BI15)</f>
-        <v>21</v>
+        <f t="shared" si="2"/>
+        <v>24</v>
       </c>
       <c r="D15" s="11">
-        <f>SUM(I15:V15)</f>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="E15" s="11">
-        <f>SUM(W15:AI15)</f>
+        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="F15" s="11">
-        <f>SUM(AJ15:AV15)</f>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>3</v>
       </c>
       <c r="G15" s="11">
-        <f>SUM(AW15:BI15)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H15" s="11">
-        <f>COUNT(I15:BI15)</f>
-        <v>17</v>
+        <f t="shared" si="7"/>
+        <v>18</v>
       </c>
       <c r="I15" s="3">
         <v>0</v>
@@ -6494,7 +6515,9 @@
       <c r="AI15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ15" s="3"/>
+      <c r="AJ15" s="3">
+        <v>3</v>
+      </c>
       <c r="AK15" s="3"/>
       <c r="AL15" s="3"/>
       <c r="AM15" s="3"/>
@@ -6526,28 +6549,28 @@
         <v>17</v>
       </c>
       <c r="C16" s="6">
-        <f>SUM(I16:BI16)</f>
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="D16" s="11">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="E16" s="11">
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
-      <c r="D16" s="11">
-        <f>SUM(I16:V16)</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="11">
-        <f>SUM(W16:AI16)</f>
-        <v>9</v>
-      </c>
       <c r="F16" s="11">
-        <f>SUM(AJ16:AV16)</f>
-        <v>0</v>
+        <f t="shared" si="5"/>
+        <v>3</v>
       </c>
       <c r="G16" s="11">
-        <f>SUM(AW16:BI16)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H16" s="11">
-        <f>COUNT(I16:BI16)</f>
-        <v>3</v>
+        <f t="shared" si="7"/>
+        <v>4</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>19</v>
@@ -6630,7 +6653,9 @@
       <c r="AI16" s="3">
         <v>3</v>
       </c>
-      <c r="AJ16" s="3"/>
+      <c r="AJ16" s="3">
+        <v>3</v>
+      </c>
       <c r="AK16" s="3"/>
       <c r="AL16" s="3"/>
       <c r="AM16" s="3"/>
@@ -6662,27 +6687,27 @@
         <v>10</v>
       </c>
       <c r="C17" s="6">
-        <f>SUM(I17:BI17)</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D17" s="11">
-        <f>SUM(I17:V17)</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="E17" s="11">
-        <f>SUM(W17:AI17)</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="F17" s="11">
-        <f>SUM(AJ17:AV17)</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G17" s="11">
-        <f>SUM(AW17:BI17)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="H17" s="11">
-        <f>COUNT(I17:BI17)</f>
+        <f t="shared" si="7"/>
         <v>2</v>
       </c>
       <c r="I17" s="3" t="s">
@@ -6766,7 +6791,9 @@
       <c r="AI17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ17" s="3"/>
+      <c r="AJ17" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK17" s="3"/>
       <c r="AL17" s="3"/>
       <c r="AM17" s="3"/>
@@ -6819,27 +6846,27 @@
         <v>46025</v>
       </c>
       <c r="J18" s="5">
-        <f t="shared" ref="J18:O18" si="2">I18+7</f>
+        <f t="shared" ref="J18:O18" si="8">I18+7</f>
         <v>46032</v>
       </c>
       <c r="K18" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>46039</v>
       </c>
       <c r="L18" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>46046</v>
       </c>
       <c r="M18" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>46053</v>
       </c>
       <c r="N18" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>46060</v>
       </c>
       <c r="O18" s="5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="8"/>
         <v>46067</v>
       </c>
       <c r="P18" s="5">
@@ -6870,159 +6897,159 @@
         <v>46109</v>
       </c>
       <c r="W18" s="5">
-        <f t="shared" ref="W18:BH18" si="3">V18+7</f>
+        <f t="shared" ref="W18:BH18" si="9">V18+7</f>
         <v>46116</v>
       </c>
       <c r="X18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46123</v>
       </c>
       <c r="Y18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46130</v>
       </c>
       <c r="Z18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46137</v>
       </c>
       <c r="AA18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46144</v>
       </c>
       <c r="AB18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46151</v>
       </c>
       <c r="AC18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46158</v>
       </c>
       <c r="AD18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46165</v>
       </c>
       <c r="AE18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46172</v>
       </c>
       <c r="AF18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46179</v>
       </c>
       <c r="AG18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46186</v>
       </c>
       <c r="AH18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46193</v>
       </c>
       <c r="AI18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46200</v>
       </c>
       <c r="AJ18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46207</v>
       </c>
       <c r="AK18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46214</v>
       </c>
       <c r="AL18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46221</v>
       </c>
       <c r="AM18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46228</v>
       </c>
       <c r="AN18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46235</v>
       </c>
       <c r="AO18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46242</v>
       </c>
       <c r="AP18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46249</v>
       </c>
       <c r="AQ18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46256</v>
       </c>
       <c r="AR18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46263</v>
       </c>
       <c r="AS18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46270</v>
       </c>
       <c r="AT18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46277</v>
       </c>
       <c r="AU18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46284</v>
       </c>
       <c r="AV18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46291</v>
       </c>
       <c r="AW18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46298</v>
       </c>
       <c r="AX18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46305</v>
       </c>
       <c r="AY18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46312</v>
       </c>
       <c r="AZ18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46319</v>
       </c>
       <c r="BA18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46326</v>
       </c>
       <c r="BB18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46333</v>
       </c>
       <c r="BC18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46340</v>
       </c>
       <c r="BD18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46347</v>
       </c>
       <c r="BE18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46354</v>
       </c>
       <c r="BF18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46361</v>
       </c>
       <c r="BG18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46368</v>
       </c>
       <c r="BH18" s="5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>46375</v>
       </c>
       <c r="BI18" s="5">
-        <f t="shared" ref="BI18" si="4">BH18+7</f>
+        <f t="shared" ref="BI18" si="10">BH18+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -7135,7 +7162,9 @@
       <c r="AI19" s="3">
         <v>3</v>
       </c>
-      <c r="AJ19" s="3"/>
+      <c r="AJ19" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK19" s="3"/>
       <c r="AL19" s="3"/>
       <c r="AM19" s="3"/>
@@ -7188,7 +7217,7 @@
       </c>
       <c r="H20" s="11">
         <f>COUNT(I20:BI20)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>19</v>
@@ -7271,7 +7300,9 @@
       <c r="AI20" s="3">
         <v>0</v>
       </c>
-      <c r="AJ20" s="3"/>
+      <c r="AJ20" s="3">
+        <v>0</v>
+      </c>
       <c r="AK20" s="3"/>
       <c r="AL20" s="3"/>
       <c r="AM20" s="3"/>
@@ -7392,23 +7423,23 @@
         <v>46032</v>
       </c>
       <c r="K23" s="5">
-        <f t="shared" ref="K23:BH23" si="5">J23+7</f>
+        <f t="shared" ref="K23:BH23" si="11">J23+7</f>
         <v>46039</v>
       </c>
       <c r="L23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46046</v>
       </c>
       <c r="M23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46053</v>
       </c>
       <c r="N23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46060</v>
       </c>
       <c r="O23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46067</v>
       </c>
       <c r="P23" s="5">
@@ -7419,179 +7450,179 @@
         <v>46074</v>
       </c>
       <c r="R23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46081</v>
       </c>
       <c r="S23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46088</v>
       </c>
       <c r="T23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46095</v>
       </c>
       <c r="U23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46102</v>
       </c>
       <c r="V23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46109</v>
       </c>
       <c r="W23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46116</v>
       </c>
       <c r="X23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46123</v>
       </c>
       <c r="Y23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46130</v>
       </c>
       <c r="Z23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46137</v>
       </c>
       <c r="AA23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46144</v>
       </c>
       <c r="AB23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46151</v>
       </c>
       <c r="AC23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46158</v>
       </c>
       <c r="AD23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46165</v>
       </c>
       <c r="AE23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46172</v>
       </c>
       <c r="AF23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46179</v>
       </c>
       <c r="AG23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46186</v>
       </c>
       <c r="AH23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46193</v>
       </c>
       <c r="AI23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46200</v>
       </c>
       <c r="AJ23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46207</v>
       </c>
       <c r="AK23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46214</v>
       </c>
       <c r="AL23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46221</v>
       </c>
       <c r="AM23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46228</v>
       </c>
       <c r="AN23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46235</v>
       </c>
       <c r="AO23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46242</v>
       </c>
       <c r="AP23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46249</v>
       </c>
       <c r="AQ23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46256</v>
       </c>
       <c r="AR23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46263</v>
       </c>
       <c r="AS23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46270</v>
       </c>
       <c r="AT23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46277</v>
       </c>
       <c r="AU23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46284</v>
       </c>
       <c r="AV23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46291</v>
       </c>
       <c r="AW23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46298</v>
       </c>
       <c r="AX23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46305</v>
       </c>
       <c r="AY23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46312</v>
       </c>
       <c r="AZ23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46319</v>
       </c>
       <c r="BA23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46326</v>
       </c>
       <c r="BB23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46333</v>
       </c>
       <c r="BC23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46340</v>
       </c>
       <c r="BD23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46347</v>
       </c>
       <c r="BE23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46354</v>
       </c>
       <c r="BF23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46361</v>
       </c>
       <c r="BG23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46368</v>
       </c>
       <c r="BH23" s="5">
-        <f t="shared" si="5"/>
+        <f t="shared" si="11"/>
         <v>46375</v>
       </c>
       <c r="BI23" s="5">
-        <f t="shared" ref="BI23" si="6">BH23+7</f>
+        <f t="shared" ref="BI23" si="12">BH23+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -7600,27 +7631,27 @@
         <v>40</v>
       </c>
       <c r="C24" s="6">
-        <f>SUM(I24:BI24)</f>
+        <f t="shared" ref="C24:C37" si="13">SUM(I24:BI24)</f>
         <v>44</v>
       </c>
       <c r="D24" s="11">
-        <f>SUM(I24:V24)</f>
+        <f t="shared" ref="D24:D37" si="14">SUM(I24:V24)</f>
         <v>20</v>
       </c>
       <c r="E24" s="11">
-        <f>SUM(W24:AI24)</f>
+        <f t="shared" ref="E24:E37" si="15">SUM(W24:AI24)</f>
         <v>24</v>
       </c>
       <c r="F24" s="11">
-        <f>SUM(AJ24:AV24)</f>
+        <f t="shared" ref="F24:F37" si="16">SUM(AJ24:AV24)</f>
         <v>0</v>
       </c>
       <c r="G24" s="11">
-        <f>SUM(AW24:BI24)</f>
+        <f t="shared" ref="G24:G37" si="17">SUM(AW24:BI24)</f>
         <v>0</v>
       </c>
       <c r="H24" s="11">
-        <f>COUNT(I24:BI24)</f>
+        <f t="shared" ref="H24:H37" si="18">COUNT(I24:BI24)</f>
         <v>23</v>
       </c>
       <c r="I24" s="3">
@@ -7704,7 +7735,9 @@
       <c r="AI24" s="3">
         <v>1</v>
       </c>
-      <c r="AJ24" s="3"/>
+      <c r="AJ24" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK24" s="3"/>
       <c r="AL24" s="3"/>
       <c r="AM24" s="3"/>
@@ -7736,28 +7769,28 @@
         <v>9</v>
       </c>
       <c r="C25" s="6">
-        <f>SUM(I25:BI25)</f>
-        <v>39</v>
+        <f t="shared" si="13"/>
+        <v>40</v>
       </c>
       <c r="D25" s="11">
-        <f>SUM(I25:V25)</f>
+        <f t="shared" si="14"/>
         <v>22</v>
       </c>
       <c r="E25" s="11">
-        <f>SUM(W25:AI25)</f>
+        <f t="shared" si="15"/>
         <v>17</v>
       </c>
       <c r="F25" s="11">
-        <f>SUM(AJ25:AV25)</f>
-        <v>0</v>
+        <f t="shared" si="16"/>
+        <v>1</v>
       </c>
       <c r="G25" s="11">
-        <f>SUM(AW25:BI25)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H25" s="11">
-        <f>COUNT(I25:BI25)</f>
-        <v>24</v>
+        <f t="shared" si="18"/>
+        <v>25</v>
       </c>
       <c r="I25" s="3">
         <v>0</v>
@@ -7840,7 +7873,9 @@
       <c r="AI25" s="3">
         <v>0</v>
       </c>
-      <c r="AJ25" s="3"/>
+      <c r="AJ25" s="3">
+        <v>1</v>
+      </c>
       <c r="AK25" s="3"/>
       <c r="AL25" s="3"/>
       <c r="AM25" s="3"/>
@@ -7872,28 +7907,28 @@
         <v>33</v>
       </c>
       <c r="C26" s="6">
-        <f>SUM(I26:BI26)</f>
-        <v>34</v>
+        <f t="shared" si="13"/>
+        <v>35</v>
       </c>
       <c r="D26" s="11">
-        <f>SUM(I26:V26)</f>
+        <f t="shared" si="14"/>
         <v>19</v>
       </c>
       <c r="E26" s="11">
-        <f>SUM(W26:AI26)</f>
+        <f t="shared" si="15"/>
         <v>15</v>
       </c>
       <c r="F26" s="11">
-        <f>SUM(AJ26:AV26)</f>
-        <v>0</v>
+        <f t="shared" si="16"/>
+        <v>1</v>
       </c>
       <c r="G26" s="11">
-        <f>SUM(AW26:BI26)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H26" s="11">
-        <f>COUNT(I26:BI26)</f>
-        <v>22</v>
+        <f t="shared" si="18"/>
+        <v>23</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>19</v>
@@ -7976,7 +8011,9 @@
       <c r="AI26" s="3">
         <v>1</v>
       </c>
-      <c r="AJ26" s="3"/>
+      <c r="AJ26" s="3">
+        <v>1</v>
+      </c>
       <c r="AK26" s="3"/>
       <c r="AL26" s="3"/>
       <c r="AM26" s="3"/>
@@ -8008,28 +8045,28 @@
         <v>5</v>
       </c>
       <c r="C27" s="6">
-        <f>SUM(I27:BI27)</f>
-        <v>31</v>
+        <f t="shared" si="13"/>
+        <v>32</v>
       </c>
       <c r="D27" s="11">
-        <f>SUM(I27:V27)</f>
+        <f t="shared" si="14"/>
         <v>19</v>
       </c>
       <c r="E27" s="11">
-        <f>SUM(W27:AI27)</f>
+        <f t="shared" si="15"/>
         <v>12</v>
       </c>
       <c r="F27" s="11">
-        <f>SUM(AJ27:AV27)</f>
-        <v>0</v>
+        <f t="shared" si="16"/>
+        <v>1</v>
       </c>
       <c r="G27" s="11">
-        <f>SUM(AW27:BI27)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H27" s="11">
-        <f>COUNT(I27:BI27)</f>
-        <v>23</v>
+        <f t="shared" si="18"/>
+        <v>24</v>
       </c>
       <c r="I27" s="3">
         <v>4</v>
@@ -8112,7 +8149,9 @@
       <c r="AI27" s="3">
         <v>1</v>
       </c>
-      <c r="AJ27" s="3"/>
+      <c r="AJ27" s="3">
+        <v>1</v>
+      </c>
       <c r="AK27" s="3"/>
       <c r="AL27" s="3"/>
       <c r="AM27" s="3"/>
@@ -8144,27 +8183,27 @@
         <v>11</v>
       </c>
       <c r="C28" s="6">
-        <f>SUM(I28:BI28)</f>
+        <f t="shared" si="13"/>
         <v>28</v>
       </c>
       <c r="D28" s="11">
-        <f>SUM(I28:V28)</f>
+        <f t="shared" si="14"/>
         <v>14</v>
       </c>
       <c r="E28" s="11">
-        <f>SUM(W28:AI28)</f>
+        <f t="shared" si="15"/>
         <v>14</v>
       </c>
       <c r="F28" s="11">
-        <f>SUM(AJ28:AV28)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G28" s="11">
-        <f>SUM(AW28:BI28)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H28" s="11">
-        <f>COUNT(I28:BI28)</f>
+        <f t="shared" si="18"/>
         <v>20</v>
       </c>
       <c r="I28" s="3">
@@ -8248,7 +8287,9 @@
       <c r="AI28" s="3">
         <v>1</v>
       </c>
-      <c r="AJ28" s="3"/>
+      <c r="AJ28" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK28" s="3"/>
       <c r="AL28" s="3"/>
       <c r="AM28" s="3"/>
@@ -8280,28 +8321,28 @@
         <v>3</v>
       </c>
       <c r="C29" s="6">
-        <f>SUM(I29:BI29)</f>
-        <v>27</v>
+        <f t="shared" si="13"/>
+        <v>28</v>
       </c>
       <c r="D29" s="11">
-        <f>SUM(I29:V29)</f>
+        <f t="shared" si="14"/>
         <v>10</v>
       </c>
       <c r="E29" s="11">
-        <f>SUM(W29:AI29)</f>
+        <f t="shared" si="15"/>
         <v>17</v>
       </c>
       <c r="F29" s="11">
-        <f>SUM(AJ29:AV29)</f>
-        <v>0</v>
+        <f t="shared" si="16"/>
+        <v>1</v>
       </c>
       <c r="G29" s="11">
-        <f>SUM(AW29:BI29)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H29" s="11">
-        <f>COUNT(I29:BI29)</f>
-        <v>23</v>
+        <f t="shared" si="18"/>
+        <v>24</v>
       </c>
       <c r="I29" s="3">
         <v>1</v>
@@ -8384,7 +8425,9 @@
       <c r="AI29" s="3">
         <v>0</v>
       </c>
-      <c r="AJ29" s="3"/>
+      <c r="AJ29" s="3">
+        <v>1</v>
+      </c>
       <c r="AK29" s="3"/>
       <c r="AL29" s="3"/>
       <c r="AM29" s="3"/>
@@ -8416,28 +8459,28 @@
         <v>18</v>
       </c>
       <c r="C30" s="6">
-        <f>SUM(I30:BI30)</f>
+        <f t="shared" si="13"/>
         <v>23</v>
       </c>
       <c r="D30" s="11">
-        <f>SUM(I30:V30)</f>
+        <f t="shared" si="14"/>
         <v>13</v>
       </c>
       <c r="E30" s="11">
-        <f>SUM(W30:AI30)</f>
+        <f t="shared" si="15"/>
         <v>10</v>
       </c>
       <c r="F30" s="11">
-        <f>SUM(AJ30:AV30)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G30" s="11">
-        <f>SUM(AW30:BI30)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H30" s="11">
-        <f>COUNT(I30:BI30)</f>
-        <v>25</v>
+        <f t="shared" si="18"/>
+        <v>26</v>
       </c>
       <c r="I30" s="3">
         <v>0</v>
@@ -8520,7 +8563,9 @@
       <c r="AI30" s="3">
         <v>0</v>
       </c>
-      <c r="AJ30" s="3"/>
+      <c r="AJ30" s="3">
+        <v>0</v>
+      </c>
       <c r="AK30" s="3"/>
       <c r="AL30" s="3"/>
       <c r="AM30" s="3"/>
@@ -8552,28 +8597,28 @@
         <v>35</v>
       </c>
       <c r="C31" s="6">
-        <f>SUM(I31:BI31)</f>
-        <v>23</v>
+        <f t="shared" si="13"/>
+        <v>24</v>
       </c>
       <c r="D31" s="11">
-        <f>SUM(I31:V31)</f>
+        <f t="shared" si="14"/>
         <v>11</v>
       </c>
       <c r="E31" s="11">
-        <f>SUM(W31:AI31)</f>
+        <f t="shared" si="15"/>
         <v>12</v>
       </c>
       <c r="F31" s="11">
-        <f>SUM(AJ31:AV31)</f>
-        <v>0</v>
+        <f t="shared" si="16"/>
+        <v>1</v>
       </c>
       <c r="G31" s="11">
-        <f>SUM(AW31:BI31)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H31" s="11">
-        <f>COUNT(I31:BI31)</f>
-        <v>26</v>
+        <f t="shared" si="18"/>
+        <v>27</v>
       </c>
       <c r="I31" s="3">
         <v>2</v>
@@ -8656,7 +8701,9 @@
       <c r="AI31" s="3">
         <v>0</v>
       </c>
-      <c r="AJ31" s="3"/>
+      <c r="AJ31" s="3">
+        <v>1</v>
+      </c>
       <c r="AK31" s="3"/>
       <c r="AL31" s="3"/>
       <c r="AM31" s="3"/>
@@ -8688,27 +8735,27 @@
         <v>15</v>
       </c>
       <c r="C32" s="6">
-        <f>SUM(I32:BI32)</f>
+        <f t="shared" si="13"/>
         <v>19</v>
       </c>
       <c r="D32" s="11">
-        <f>SUM(I32:V32)</f>
+        <f t="shared" si="14"/>
         <v>8</v>
       </c>
       <c r="E32" s="11">
-        <f>SUM(W32:AI32)</f>
+        <f t="shared" si="15"/>
         <v>11</v>
       </c>
       <c r="F32" s="11">
-        <f>SUM(AJ32:AV32)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G32" s="11">
-        <f>SUM(AW32:BI32)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H32" s="11">
-        <f>COUNT(I32:BI32)</f>
+        <f t="shared" si="18"/>
         <v>14</v>
       </c>
       <c r="I32" s="3" t="s">
@@ -8792,7 +8839,9 @@
       <c r="AI32" s="3">
         <v>2</v>
       </c>
-      <c r="AJ32" s="3"/>
+      <c r="AJ32" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK32" s="3"/>
       <c r="AL32" s="3"/>
       <c r="AM32" s="3"/>
@@ -8824,28 +8873,28 @@
         <v>7</v>
       </c>
       <c r="C33" s="6">
-        <f>SUM(I33:BI33)</f>
+        <f t="shared" si="13"/>
         <v>16</v>
       </c>
       <c r="D33" s="11">
-        <f>SUM(I33:V33)</f>
+        <f t="shared" si="14"/>
         <v>10</v>
       </c>
       <c r="E33" s="11">
-        <f>SUM(W33:AI33)</f>
+        <f t="shared" si="15"/>
         <v>6</v>
       </c>
       <c r="F33" s="11">
-        <f>SUM(AJ33:AV33)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G33" s="11">
-        <f>SUM(AW33:BI33)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H33" s="11">
-        <f>COUNT(I33:BI33)</f>
-        <v>19</v>
+        <f t="shared" si="18"/>
+        <v>20</v>
       </c>
       <c r="I33" s="3">
         <v>2</v>
@@ -8928,7 +8977,9 @@
       <c r="AI33" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ33" s="3"/>
+      <c r="AJ33" s="3">
+        <v>0</v>
+      </c>
       <c r="AK33" s="3"/>
       <c r="AL33" s="3"/>
       <c r="AM33" s="3"/>
@@ -8960,28 +9011,28 @@
         <v>6</v>
       </c>
       <c r="C34" s="6">
-        <f>SUM(I34:BI34)</f>
-        <v>7</v>
+        <f t="shared" si="13"/>
+        <v>8</v>
       </c>
       <c r="D34" s="11">
-        <f>SUM(I34:V34)</f>
+        <f t="shared" si="14"/>
         <v>4</v>
       </c>
       <c r="E34" s="11">
-        <f>SUM(W34:AI34)</f>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
       <c r="F34" s="11">
-        <f>SUM(AJ34:AV34)</f>
-        <v>0</v>
+        <f t="shared" si="16"/>
+        <v>1</v>
       </c>
       <c r="G34" s="11">
-        <f>SUM(AW34:BI34)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H34" s="11">
-        <f>COUNT(I34:BI34)</f>
-        <v>16</v>
+        <f t="shared" si="18"/>
+        <v>17</v>
       </c>
       <c r="I34" s="3">
         <v>0</v>
@@ -9064,7 +9115,9 @@
       <c r="AI34" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ34" s="3"/>
+      <c r="AJ34" s="3">
+        <v>1</v>
+      </c>
       <c r="AK34" s="3"/>
       <c r="AL34" s="3"/>
       <c r="AM34" s="3"/>
@@ -9096,28 +9149,28 @@
         <v>36</v>
       </c>
       <c r="C35" s="6">
-        <f>SUM(I35:BI35)</f>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="D35" s="11">
-        <f>SUM(I35:V35)</f>
+        <f t="shared" si="14"/>
         <v>3</v>
       </c>
       <c r="E35" s="11">
-        <f>SUM(W35:AI35)</f>
+        <f t="shared" si="15"/>
         <v>2</v>
       </c>
       <c r="F35" s="11">
-        <f>SUM(AJ35:AV35)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G35" s="11">
-        <f>SUM(AW35:BI35)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H35" s="11">
-        <f>COUNT(I35:BI35)</f>
-        <v>16</v>
+        <f t="shared" si="18"/>
+        <v>17</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>19</v>
@@ -9200,7 +9253,9 @@
       <c r="AI35" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ35" s="3"/>
+      <c r="AJ35" s="3">
+        <v>0</v>
+      </c>
       <c r="AK35" s="3"/>
       <c r="AL35" s="3"/>
       <c r="AM35" s="3"/>
@@ -9232,28 +9287,28 @@
         <v>17</v>
       </c>
       <c r="C36" s="6">
-        <f>SUM(I36:BI36)</f>
+        <f t="shared" si="13"/>
         <v>3</v>
       </c>
       <c r="D36" s="11">
-        <f>SUM(I36:V36)</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="E36" s="11">
-        <f>SUM(W36:AI36)</f>
+        <f t="shared" si="15"/>
         <v>3</v>
       </c>
       <c r="F36" s="11">
-        <f>SUM(AJ36:AV36)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G36" s="11">
-        <f>SUM(AW36:BI36)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H36" s="11">
-        <f>COUNT(I36:BI36)</f>
-        <v>4</v>
+        <f t="shared" si="18"/>
+        <v>5</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>19</v>
@@ -9336,7 +9391,9 @@
       <c r="AI36" s="3">
         <v>1</v>
       </c>
-      <c r="AJ36" s="3"/>
+      <c r="AJ36" s="3">
+        <v>0</v>
+      </c>
       <c r="AK36" s="3"/>
       <c r="AL36" s="3"/>
       <c r="AM36" s="3"/>
@@ -9368,27 +9425,27 @@
         <v>10</v>
       </c>
       <c r="C37" s="6">
-        <f>SUM(I37:BI37)</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="D37" s="11">
-        <f>SUM(I37:V37)</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="E37" s="11">
-        <f>SUM(W37:AI37)</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F37" s="11">
-        <f>SUM(AJ37:AV37)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G37" s="11">
-        <f>SUM(AW37:BI37)</f>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="H37" s="11">
-        <f>COUNT(I37:BI37)</f>
+        <f t="shared" si="18"/>
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
@@ -9472,7 +9529,9 @@
       <c r="AI37" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AJ37" s="3"/>
+      <c r="AJ37" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AK37" s="3"/>
       <c r="AL37" s="3"/>
       <c r="AM37" s="3"/>
@@ -9529,23 +9588,23 @@
         <v>46032</v>
       </c>
       <c r="K38" s="5">
-        <f t="shared" ref="K38:BH38" si="7">J38+7</f>
+        <f t="shared" ref="K38:BH38" si="19">J38+7</f>
         <v>46039</v>
       </c>
       <c r="L38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46046</v>
       </c>
       <c r="M38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46053</v>
       </c>
       <c r="N38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46060</v>
       </c>
       <c r="O38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46067</v>
       </c>
       <c r="P38" s="5">
@@ -9556,179 +9615,179 @@
         <v>46074</v>
       </c>
       <c r="R38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46081</v>
       </c>
       <c r="S38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46088</v>
       </c>
       <c r="T38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46095</v>
       </c>
       <c r="U38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46102</v>
       </c>
       <c r="V38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46109</v>
       </c>
       <c r="W38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46116</v>
       </c>
       <c r="X38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46123</v>
       </c>
       <c r="Y38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46130</v>
       </c>
       <c r="Z38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46137</v>
       </c>
       <c r="AA38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46144</v>
       </c>
       <c r="AB38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46151</v>
       </c>
       <c r="AC38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46158</v>
       </c>
       <c r="AD38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46165</v>
       </c>
       <c r="AE38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46172</v>
       </c>
       <c r="AF38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46179</v>
       </c>
       <c r="AG38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46186</v>
       </c>
       <c r="AH38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46193</v>
       </c>
       <c r="AI38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46200</v>
       </c>
       <c r="AJ38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46207</v>
       </c>
       <c r="AK38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46214</v>
       </c>
       <c r="AL38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46221</v>
       </c>
       <c r="AM38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46228</v>
       </c>
       <c r="AN38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46235</v>
       </c>
       <c r="AO38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46242</v>
       </c>
       <c r="AP38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46249</v>
       </c>
       <c r="AQ38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46256</v>
       </c>
       <c r="AR38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46263</v>
       </c>
       <c r="AS38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46270</v>
       </c>
       <c r="AT38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46277</v>
       </c>
       <c r="AU38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46284</v>
       </c>
       <c r="AV38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46291</v>
       </c>
       <c r="AW38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46298</v>
       </c>
       <c r="AX38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46305</v>
       </c>
       <c r="AY38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46312</v>
       </c>
       <c r="AZ38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46319</v>
       </c>
       <c r="BA38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46326</v>
       </c>
       <c r="BB38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46333</v>
       </c>
       <c r="BC38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46340</v>
       </c>
       <c r="BD38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46347</v>
       </c>
       <c r="BE38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46354</v>
       </c>
       <c r="BF38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46361</v>
       </c>
       <c r="BG38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46368</v>
       </c>
       <c r="BH38" s="5">
-        <f t="shared" si="7"/>
+        <f t="shared" si="19"/>
         <v>46375</v>
       </c>
       <c r="BI38" s="5">
-        <f t="shared" ref="BI38" si="8">BH38+7</f>
+        <f t="shared" ref="BI38" si="20">BH38+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -9741,24 +9800,24 @@
         <v>0</v>
       </c>
       <c r="D39" s="11">
-        <f t="shared" ref="D39:D40" si="9">SUM(I39:V39)</f>
+        <f t="shared" ref="D39:D40" si="21">SUM(I39:V39)</f>
         <v>0</v>
       </c>
       <c r="E39" s="11">
-        <f t="shared" ref="E39:E40" si="10">SUM(W39:AI39)</f>
+        <f t="shared" ref="E39:E40" si="22">SUM(W39:AI39)</f>
         <v>0</v>
       </c>
       <c r="F39" s="11">
-        <f t="shared" ref="F39:F40" si="11">SUM(AJ39:AV39)</f>
+        <f t="shared" ref="F39:F40" si="23">SUM(AJ39:AV39)</f>
         <v>0</v>
       </c>
       <c r="G39" s="11">
-        <f t="shared" ref="G39:G40" si="12">SUM(AW39:BI39)</f>
+        <f t="shared" ref="G39:G40" si="24">SUM(AW39:BI39)</f>
         <v>0</v>
       </c>
       <c r="H39" s="11">
-        <f t="shared" ref="H39:H40" si="13">COUNT(I39:BI39)</f>
-        <v>22</v>
+        <f t="shared" ref="H39:H40" si="25">COUNT(I39:BI39)</f>
+        <v>23</v>
       </c>
       <c r="I39" s="3">
         <v>0</v>
@@ -9841,7 +9900,9 @@
       <c r="AI39" s="3">
         <v>0</v>
       </c>
-      <c r="AJ39" s="3"/>
+      <c r="AJ39" s="3">
+        <v>0</v>
+      </c>
       <c r="AK39" s="3"/>
       <c r="AL39" s="3"/>
       <c r="AM39" s="3"/>
@@ -9877,24 +9938,24 @@
         <v>0</v>
       </c>
       <c r="D40" s="11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="E40" s="11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="F40" s="11">
-        <f t="shared" si="11"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="G40" s="11">
-        <f t="shared" si="12"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
       <c r="H40" s="11">
-        <f t="shared" si="13"/>
-        <v>20</v>
+        <f t="shared" si="25"/>
+        <v>21</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>19</v>
@@ -9977,7 +10038,9 @@
       <c r="AI40" s="3">
         <v>0</v>
       </c>
-      <c r="AJ40" s="3"/>
+      <c r="AJ40" s="3">
+        <v>0</v>
+      </c>
       <c r="AK40" s="3"/>
       <c r="AL40" s="3"/>
       <c r="AM40" s="3"/>

</xml_diff>

<commit_message>
feat: update player statistics and add new player to the dataset
</commit_message>
<xml_diff>
--- a/Pontuação 2026.xlsx
+++ b/Pontuação 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luan-\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31369FC3-FDBA-4ECA-9A02-D347394C7034}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A3CEAD-555D-4E53-9018-15E1988DF675}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="41">
   <si>
     <t>Atletas</t>
   </si>
@@ -4893,28 +4893,28 @@
         <v>40</v>
       </c>
       <c r="C4" s="6">
-        <f t="shared" ref="C4:C17" si="2">SUM(I4:BI4)</f>
+        <f>SUM(I4:BI4)</f>
         <v>53</v>
       </c>
       <c r="D4" s="11">
-        <f t="shared" ref="D4:D17" si="3">SUM(I4:V4)</f>
+        <f>SUM(I4:V4)</f>
         <v>29</v>
       </c>
       <c r="E4" s="11">
-        <f t="shared" ref="E4:E17" si="4">SUM(W4:AI4)</f>
+        <f>SUM(W4:AI4)</f>
         <v>24</v>
       </c>
       <c r="F4" s="11">
-        <f t="shared" ref="F4:F17" si="5">SUM(AJ4:AV4)</f>
+        <f>SUM(AJ4:AV4)</f>
         <v>0</v>
       </c>
       <c r="G4" s="11">
-        <f t="shared" ref="G4:G17" si="6">SUM(AW4:BI4)</f>
+        <f>SUM(AW4:BI4)</f>
         <v>0</v>
       </c>
       <c r="H4" s="11">
-        <f t="shared" ref="H4:H17" si="7">COUNT(I4:BI4)</f>
-        <v>23</v>
+        <f>COUNT(I4:BI4)</f>
+        <v>24</v>
       </c>
       <c r="I4" s="3">
         <v>3</v>
@@ -5000,7 +5000,9 @@
       <c r="AJ4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK4" s="3"/>
+      <c r="AK4" s="3">
+        <v>0</v>
+      </c>
       <c r="AL4" s="3"/>
       <c r="AM4" s="3"/>
       <c r="AN4" s="3"/>
@@ -5031,28 +5033,28 @@
         <v>9</v>
       </c>
       <c r="C5" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I5:BI5)</f>
         <v>37</v>
       </c>
       <c r="D5" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I5:V5)</f>
         <v>16</v>
       </c>
       <c r="E5" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W5:AI5)</f>
         <v>21</v>
       </c>
       <c r="F5" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ5:AV5)</f>
         <v>0</v>
       </c>
       <c r="G5" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW5:BI5)</f>
         <v>0</v>
       </c>
       <c r="H5" s="11">
-        <f t="shared" si="7"/>
-        <v>24</v>
+        <f>COUNT(I5:BI5)</f>
+        <v>25</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>19</v>
@@ -5138,7 +5140,9 @@
       <c r="AJ5" s="3">
         <v>0</v>
       </c>
-      <c r="AK5" s="3"/>
+      <c r="AK5" s="3">
+        <v>0</v>
+      </c>
       <c r="AL5" s="3"/>
       <c r="AM5" s="3"/>
       <c r="AN5" s="3"/>
@@ -5169,28 +5173,28 @@
         <v>33</v>
       </c>
       <c r="C6" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I6:BI6)</f>
         <v>37</v>
       </c>
       <c r="D6" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I6:V6)</f>
         <v>16</v>
       </c>
       <c r="E6" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W6:AI6)</f>
         <v>18</v>
       </c>
       <c r="F6" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ6:AV6)</f>
         <v>3</v>
       </c>
       <c r="G6" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW6:BI6)</f>
         <v>0</v>
       </c>
       <c r="H6" s="11">
-        <f t="shared" si="7"/>
-        <v>23</v>
+        <f>COUNT(I6:BI6)</f>
+        <v>24</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>19</v>
@@ -5276,7 +5280,9 @@
       <c r="AJ6" s="3">
         <v>3</v>
       </c>
-      <c r="AK6" s="3"/>
+      <c r="AK6" s="3">
+        <v>0</v>
+      </c>
       <c r="AL6" s="3"/>
       <c r="AM6" s="3"/>
       <c r="AN6" s="3"/>
@@ -5307,28 +5313,28 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <f t="shared" si="2"/>
-        <v>32</v>
+        <f>SUM(I7:BI7)</f>
+        <v>35</v>
       </c>
       <c r="D7" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I7:V7)</f>
         <v>14</v>
       </c>
       <c r="E7" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W7:AI7)</f>
         <v>18</v>
       </c>
       <c r="F7" s="11">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>SUM(AJ7:AV7)</f>
+        <v>3</v>
       </c>
       <c r="G7" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW7:BI7)</f>
         <v>0</v>
       </c>
       <c r="H7" s="11">
-        <f t="shared" si="7"/>
-        <v>27</v>
+        <f>COUNT(I7:BI7)</f>
+        <v>28</v>
       </c>
       <c r="I7" s="3">
         <v>3</v>
@@ -5414,7 +5420,9 @@
       <c r="AJ7" s="3">
         <v>0</v>
       </c>
-      <c r="AK7" s="3"/>
+      <c r="AK7" s="3">
+        <v>3</v>
+      </c>
       <c r="AL7" s="3"/>
       <c r="AM7" s="3"/>
       <c r="AN7" s="3"/>
@@ -5442,34 +5450,34 @@
     </row>
     <row r="8" spans="2:61" ht="14.1" customHeight="1">
       <c r="B8" s="14" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="C8" s="6">
-        <f t="shared" si="2"/>
-        <v>29</v>
+        <f>SUM(I8:BI8)</f>
+        <v>31</v>
       </c>
       <c r="D8" s="11">
-        <f t="shared" si="3"/>
-        <v>20</v>
+        <f>SUM(I8:V8)</f>
+        <v>16</v>
       </c>
       <c r="E8" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W8:AI8)</f>
         <v>9</v>
       </c>
       <c r="F8" s="11">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>SUM(AJ8:AV8)</f>
+        <v>6</v>
       </c>
       <c r="G8" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW8:BI8)</f>
         <v>0</v>
       </c>
       <c r="H8" s="11">
-        <f t="shared" si="7"/>
-        <v>18</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>19</v>
+        <f>COUNT(I8:BI8)</f>
+        <v>26</v>
+      </c>
+      <c r="I8" s="3">
+        <v>3</v>
       </c>
       <c r="J8" s="3">
         <v>0</v>
@@ -5481,64 +5489,64 @@
         <v>3</v>
       </c>
       <c r="M8" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3">
         <v>0</v>
       </c>
-      <c r="O8" s="3" t="s">
-        <v>19</v>
+      <c r="O8" s="3">
+        <v>3</v>
       </c>
       <c r="P8" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>0</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R8" s="3">
+        <v>0</v>
       </c>
       <c r="S8" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T8" s="3">
         <v>3</v>
       </c>
       <c r="U8" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V8" s="3">
         <v>3</v>
       </c>
-      <c r="W8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="X8" s="3" t="s">
-        <v>19</v>
+      <c r="W8" s="3">
+        <v>0</v>
+      </c>
+      <c r="X8" s="3">
+        <v>0</v>
       </c>
       <c r="Y8" s="3">
         <v>3</v>
       </c>
       <c r="Z8" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB8" s="3">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="AA8" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AC8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AD8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE8" s="3" t="s">
-        <v>19</v>
+      <c r="AD8" s="3">
+        <v>3</v>
+      </c>
+      <c r="AE8" s="3">
+        <v>0</v>
       </c>
       <c r="AF8" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AG8" s="3">
         <v>0</v>
@@ -5546,13 +5554,15 @@
       <c r="AH8" s="3">
         <v>0</v>
       </c>
-      <c r="AI8" s="3" t="s">
-        <v>19</v>
+      <c r="AI8" s="3">
+        <v>0</v>
       </c>
       <c r="AJ8" s="3">
-        <v>0</v>
-      </c>
-      <c r="AK8" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="AK8" s="3">
+        <v>3</v>
+      </c>
       <c r="AL8" s="3"/>
       <c r="AM8" s="3"/>
       <c r="AN8" s="3"/>
@@ -5580,34 +5590,34 @@
     </row>
     <row r="9" spans="2:61" ht="14.1" customHeight="1">
       <c r="B9" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="6">
+        <f>SUM(I9:BI9)</f>
+        <v>29</v>
+      </c>
+      <c r="D9" s="11">
+        <f>SUM(I9:V9)</f>
+        <v>20</v>
+      </c>
+      <c r="E9" s="11">
+        <f>SUM(W9:AI9)</f>
+        <v>9</v>
+      </c>
+      <c r="F9" s="11">
+        <f>SUM(AJ9:AV9)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="11">
+        <f>SUM(AW9:BI9)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="11">
+        <f>COUNT(I9:BI9)</f>
         <v>18</v>
       </c>
-      <c r="C9" s="6">
-        <f t="shared" si="2"/>
-        <v>28</v>
-      </c>
-      <c r="D9" s="11">
-        <f t="shared" si="3"/>
-        <v>10</v>
-      </c>
-      <c r="E9" s="11">
-        <f t="shared" si="4"/>
-        <v>18</v>
-      </c>
-      <c r="F9" s="11">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="G9" s="11">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="11">
-        <f t="shared" si="7"/>
-        <v>26</v>
-      </c>
-      <c r="I9" s="3">
-        <v>3</v>
+      <c r="I9" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="J9" s="3">
         <v>0</v>
@@ -5616,81 +5626,83 @@
         <v>1</v>
       </c>
       <c r="L9" s="3">
-        <v>0</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="M9" s="3">
+        <v>3</v>
       </c>
       <c r="N9" s="3">
-        <v>3</v>
-      </c>
-      <c r="O9" s="3">
-        <v>3</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P9" s="3">
+        <v>1</v>
       </c>
       <c r="Q9" s="3">
         <v>0</v>
       </c>
-      <c r="R9" s="3">
-        <v>0</v>
+      <c r="R9" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="S9" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T9" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U9" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V9" s="3">
-        <v>0</v>
-      </c>
-      <c r="W9" s="3">
-        <v>0</v>
-      </c>
-      <c r="X9" s="3">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="X9" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Y9" s="3">
         <v>3</v>
       </c>
       <c r="Z9" s="3">
-        <v>3</v>
-      </c>
-      <c r="AA9" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="AA9" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AB9" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="3">
-        <v>3</v>
-      </c>
-      <c r="AD9" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE9" s="3">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="AC9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE9" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AF9" s="3">
         <v>3</v>
       </c>
       <c r="AG9" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AH9" s="3">
         <v>0</v>
       </c>
-      <c r="AI9" s="3">
-        <v>0</v>
+      <c r="AI9" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AJ9" s="3">
         <v>0</v>
       </c>
-      <c r="AK9" s="3"/>
+      <c r="AK9" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
       <c r="AN9" s="3"/>
@@ -5718,70 +5730,70 @@
     </row>
     <row r="10" spans="2:61" ht="14.1" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C10" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I10:BI10)</f>
         <v>28</v>
       </c>
       <c r="D10" s="11">
-        <f t="shared" si="3"/>
-        <v>13</v>
+        <f>SUM(I10:V10)</f>
+        <v>10</v>
       </c>
       <c r="E10" s="11">
-        <f t="shared" si="4"/>
-        <v>15</v>
+        <f>SUM(W10:AI10)</f>
+        <v>18</v>
       </c>
       <c r="F10" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ10:AV10)</f>
         <v>0</v>
       </c>
       <c r="G10" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW10:BI10)</f>
         <v>0</v>
       </c>
       <c r="H10" s="11">
-        <f t="shared" si="7"/>
-        <v>15</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>19</v>
+        <f>COUNT(I10:BI10)</f>
+        <v>27</v>
+      </c>
+      <c r="I10" s="3">
+        <v>3</v>
       </c>
       <c r="J10" s="3">
-        <v>3</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="K10" s="3">
+        <v>1</v>
+      </c>
+      <c r="L10" s="3">
+        <v>0</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="N10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="P10" s="3">
-        <v>1</v>
+      <c r="N10" s="3">
+        <v>3</v>
+      </c>
+      <c r="O10" s="3">
+        <v>3</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Q10" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R10" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S10" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T10" s="3">
         <v>0</v>
       </c>
-      <c r="U10" s="3" t="s">
-        <v>19</v>
+      <c r="U10" s="3">
+        <v>0</v>
       </c>
       <c r="V10" s="3">
         <v>0</v>
@@ -5790,45 +5802,47 @@
         <v>0</v>
       </c>
       <c r="X10" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y10" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="Y10" s="3">
+        <v>3</v>
       </c>
       <c r="Z10" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AB10" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="AA10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="3">
+        <v>0</v>
       </c>
       <c r="AC10" s="3">
         <v>3</v>
       </c>
-      <c r="AD10" s="3" t="s">
-        <v>19</v>
+      <c r="AD10" s="3">
+        <v>0</v>
       </c>
       <c r="AE10" s="3">
         <v>3</v>
       </c>
       <c r="AF10" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG10" s="3">
         <v>3</v>
       </c>
-      <c r="AH10" s="3" t="s">
-        <v>19</v>
+      <c r="AH10" s="3">
+        <v>0</v>
       </c>
       <c r="AI10" s="3">
-        <v>3</v>
-      </c>
-      <c r="AJ10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AK10" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AK10" s="3">
+        <v>0</v>
+      </c>
       <c r="AL10" s="3"/>
       <c r="AM10" s="3"/>
       <c r="AN10" s="3"/>
@@ -5856,43 +5870,43 @@
     </row>
     <row r="11" spans="2:61" ht="14.1" customHeight="1">
       <c r="B11" s="14" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C11" s="6">
-        <f t="shared" si="2"/>
-        <v>26</v>
+        <f>SUM(I11:BI11)</f>
+        <v>28</v>
       </c>
       <c r="D11" s="11">
-        <f t="shared" si="3"/>
-        <v>17</v>
+        <f>SUM(I11:V11)</f>
+        <v>13</v>
       </c>
       <c r="E11" s="11">
-        <f t="shared" si="4"/>
-        <v>9</v>
+        <f>SUM(W11:AI11)</f>
+        <v>15</v>
       </c>
       <c r="F11" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ11:AV11)</f>
         <v>0</v>
       </c>
       <c r="G11" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW11:BI11)</f>
         <v>0</v>
       </c>
       <c r="H11" s="11">
-        <f t="shared" si="7"/>
-        <v>20</v>
-      </c>
-      <c r="I11" s="3">
-        <v>3</v>
+        <f>COUNT(I11:BI11)</f>
+        <v>15</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="J11" s="3">
         <v>3</v>
       </c>
-      <c r="K11" s="3">
-        <v>1</v>
-      </c>
-      <c r="L11" s="3">
-        <v>3</v>
+      <c r="K11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>19</v>
@@ -5912,8 +5926,8 @@
       <c r="R11" s="3">
         <v>3</v>
       </c>
-      <c r="S11" s="3" t="s">
-        <v>19</v>
+      <c r="S11" s="3">
+        <v>3</v>
       </c>
       <c r="T11" s="3">
         <v>0</v>
@@ -5930,43 +5944,45 @@
       <c r="X11" s="3">
         <v>3</v>
       </c>
-      <c r="Y11" s="3">
-        <v>0</v>
+      <c r="Y11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="Z11" s="3">
         <v>0</v>
       </c>
-      <c r="AA11" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB11" s="3">
-        <v>0</v>
+      <c r="AA11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB11" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AC11" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD11" s="3">
-        <v>3</v>
-      </c>
-      <c r="AE11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AF11" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="AD11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE11" s="3">
+        <v>3</v>
+      </c>
+      <c r="AF11" s="3">
+        <v>0</v>
       </c>
       <c r="AG11" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="3">
-        <v>3</v>
-      </c>
-      <c r="AI11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AJ11" s="3">
-        <v>0</v>
-      </c>
-      <c r="AK11" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="AH11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI11" s="3">
+        <v>3</v>
+      </c>
+      <c r="AJ11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AK11" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
       <c r="AN11" s="3"/>
@@ -5994,76 +6010,76 @@
     </row>
     <row r="12" spans="2:61" ht="14.1" customHeight="1">
       <c r="B12" s="14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="6">
-        <f t="shared" si="2"/>
-        <v>28</v>
+        <f>SUM(I12:BI12)</f>
+        <v>27</v>
       </c>
       <c r="D12" s="11">
-        <f t="shared" si="3"/>
-        <v>16</v>
+        <f>SUM(I12:V12)</f>
+        <v>9</v>
       </c>
       <c r="E12" s="11">
-        <f t="shared" si="4"/>
-        <v>9</v>
+        <f>SUM(W12:AI12)</f>
+        <v>12</v>
       </c>
       <c r="F12" s="11">
-        <f t="shared" si="5"/>
-        <v>3</v>
+        <f>SUM(AJ12:AV12)</f>
+        <v>6</v>
       </c>
       <c r="G12" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW12:BI12)</f>
         <v>0</v>
       </c>
       <c r="H12" s="11">
-        <f t="shared" si="7"/>
-        <v>25</v>
+        <f>COUNT(I12:BI12)</f>
+        <v>19</v>
       </c>
       <c r="I12" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3">
         <v>0</v>
       </c>
-      <c r="K12" s="3">
-        <v>1</v>
+      <c r="K12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="L12" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M12" s="3">
-        <v>0</v>
-      </c>
-      <c r="N12" s="3">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="O12" s="3">
-        <v>3</v>
-      </c>
-      <c r="P12" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="P12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>3</v>
       </c>
       <c r="R12" s="3">
         <v>0</v>
       </c>
-      <c r="S12" s="3">
-        <v>0</v>
-      </c>
-      <c r="T12" s="3">
-        <v>3</v>
+      <c r="S12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="U12" s="3">
-        <v>0</v>
-      </c>
-      <c r="V12" s="3">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="V12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="W12" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X12" s="3">
         <v>0</v>
@@ -6072,39 +6088,41 @@
         <v>3</v>
       </c>
       <c r="Z12" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA12" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AC12" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="AB12" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="3">
+        <v>3</v>
       </c>
       <c r="AD12" s="3">
-        <v>3</v>
-      </c>
-      <c r="AE12" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="AE12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AF12" s="3">
         <v>0</v>
       </c>
-      <c r="AG12" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH12" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI12" s="3">
-        <v>0</v>
+      <c r="AG12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AH12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI12" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AJ12" s="3">
         <v>3</v>
       </c>
-      <c r="AK12" s="3"/>
+      <c r="AK12" s="3">
+        <v>3</v>
+      </c>
       <c r="AL12" s="3"/>
       <c r="AM12" s="3"/>
       <c r="AN12" s="3"/>
@@ -6132,55 +6150,55 @@
     </row>
     <row r="13" spans="2:61" ht="14.1" customHeight="1">
       <c r="B13" s="14" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C13" s="6">
-        <f t="shared" si="2"/>
-        <v>25</v>
+        <f>SUM(I13:BI13)</f>
+        <v>26</v>
       </c>
       <c r="D13" s="11">
-        <f t="shared" si="3"/>
-        <v>13</v>
+        <f>SUM(I13:V13)</f>
+        <v>17</v>
       </c>
       <c r="E13" s="11">
-        <f t="shared" si="4"/>
-        <v>12</v>
+        <f>SUM(W13:AI13)</f>
+        <v>9</v>
       </c>
       <c r="F13" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ13:AV13)</f>
         <v>0</v>
       </c>
       <c r="G13" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW13:BI13)</f>
         <v>0</v>
       </c>
       <c r="H13" s="11">
-        <f t="shared" si="7"/>
+        <f>COUNT(I13:BI13)</f>
         <v>21</v>
       </c>
       <c r="I13" s="3">
-        <v>0</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="J13" s="3">
+        <v>3</v>
       </c>
       <c r="K13" s="3">
         <v>1</v>
       </c>
       <c r="L13" s="3">
-        <v>0</v>
-      </c>
-      <c r="M13" s="3">
-        <v>0</v>
-      </c>
-      <c r="N13" s="3">
-        <v>0</v>
-      </c>
-      <c r="O13" s="3">
-        <v>3</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P13" s="3">
+        <v>1</v>
       </c>
       <c r="Q13" s="3">
         <v>3</v>
@@ -6188,17 +6206,17 @@
       <c r="R13" s="3">
         <v>3</v>
       </c>
-      <c r="S13" s="3">
-        <v>0</v>
+      <c r="S13" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="T13" s="3">
         <v>0</v>
       </c>
-      <c r="U13" s="3">
-        <v>3</v>
-      </c>
-      <c r="V13" s="3" t="s">
-        <v>19</v>
+      <c r="U13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="V13" s="3">
+        <v>0</v>
       </c>
       <c r="W13" s="3">
         <v>0</v>
@@ -6210,39 +6228,41 @@
         <v>0</v>
       </c>
       <c r="Z13" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA13" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB13" s="3">
         <v>0</v>
       </c>
-      <c r="AC13" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AD13" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE13" s="3">
-        <v>3</v>
-      </c>
-      <c r="AF13" s="3">
-        <v>0</v>
+      <c r="AC13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="3">
+        <v>3</v>
+      </c>
+      <c r="AE13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AF13" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AG13" s="3">
         <v>0</v>
       </c>
-      <c r="AH13" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI13" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ13" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AK13" s="3"/>
+      <c r="AH13" s="3">
+        <v>3</v>
+      </c>
+      <c r="AI13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AJ13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AK13" s="3">
+        <v>0</v>
+      </c>
       <c r="AL13" s="3"/>
       <c r="AM13" s="3"/>
       <c r="AN13" s="3"/>
@@ -6270,37 +6290,37 @@
     </row>
     <row r="14" spans="2:61" ht="14.1" customHeight="1">
       <c r="B14" s="14" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C14" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I14:BI14)</f>
         <v>25</v>
       </c>
       <c r="D14" s="11">
-        <f t="shared" si="3"/>
-        <v>10</v>
+        <f>SUM(I14:V14)</f>
+        <v>13</v>
       </c>
       <c r="E14" s="11">
-        <f t="shared" si="4"/>
-        <v>15</v>
+        <f>SUM(W14:AI14)</f>
+        <v>12</v>
       </c>
       <c r="F14" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ14:AV14)</f>
         <v>0</v>
       </c>
       <c r="G14" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW14:BI14)</f>
         <v>0</v>
       </c>
       <c r="H14" s="11">
-        <f t="shared" si="7"/>
-        <v>24</v>
+        <f>COUNT(I14:BI14)</f>
+        <v>22</v>
       </c>
       <c r="I14" s="3">
         <v>0</v>
       </c>
-      <c r="J14" s="3">
-        <v>0</v>
+      <c r="J14" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="K14" s="3">
         <v>1</v>
@@ -6320,67 +6340,69 @@
       <c r="P14" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Q14" s="3" t="s">
-        <v>19</v>
+      <c r="Q14" s="3">
+        <v>3</v>
       </c>
       <c r="R14" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S14" s="3">
         <v>0</v>
       </c>
       <c r="T14" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="U14" s="3">
-        <v>0</v>
-      </c>
-      <c r="V14" s="3">
-        <v>3</v>
+        <v>3</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="W14" s="3">
         <v>0</v>
       </c>
       <c r="X14" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y14" s="3">
-        <v>3</v>
-      </c>
-      <c r="Z14" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="Z14" s="3">
+        <v>3</v>
       </c>
       <c r="AA14" s="3">
         <v>3</v>
       </c>
       <c r="AB14" s="3">
-        <v>3</v>
-      </c>
-      <c r="AC14" s="3">
-        <v>3</v>
-      </c>
-      <c r="AD14" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="AC14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE14" s="3">
+        <v>3</v>
       </c>
       <c r="AF14" s="3">
         <v>0</v>
       </c>
       <c r="AG14" s="3">
-        <v>3</v>
-      </c>
-      <c r="AH14" s="3">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="AH14" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AI14" s="3">
         <v>0</v>
       </c>
-      <c r="AJ14" s="3">
-        <v>0</v>
-      </c>
-      <c r="AK14" s="3"/>
+      <c r="AJ14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AK14" s="3">
+        <v>0</v>
+      </c>
       <c r="AL14" s="3"/>
       <c r="AM14" s="3"/>
       <c r="AN14" s="3"/>
@@ -6408,76 +6430,76 @@
     </row>
     <row r="15" spans="2:61" ht="14.1" customHeight="1">
       <c r="B15" s="14" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C15" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I15:BI15)</f>
+        <v>25</v>
+      </c>
+      <c r="D15" s="11">
+        <f>SUM(I15:V15)</f>
+        <v>10</v>
+      </c>
+      <c r="E15" s="11">
+        <f>SUM(W15:AI15)</f>
+        <v>15</v>
+      </c>
+      <c r="F15" s="11">
+        <f>SUM(AJ15:AV15)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="11">
+        <f>SUM(AW15:BI15)</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="11">
+        <f>COUNT(I15:BI15)</f>
         <v>24</v>
       </c>
-      <c r="D15" s="11">
-        <f t="shared" si="3"/>
-        <v>9</v>
-      </c>
-      <c r="E15" s="11">
-        <f t="shared" si="4"/>
-        <v>12</v>
-      </c>
-      <c r="F15" s="11">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="G15" s="11">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="H15" s="11">
-        <f t="shared" si="7"/>
-        <v>18</v>
-      </c>
       <c r="I15" s="3">
         <v>0</v>
       </c>
       <c r="J15" s="3">
         <v>0</v>
       </c>
-      <c r="K15" s="3" t="s">
-        <v>19</v>
+      <c r="K15" s="3">
+        <v>1</v>
       </c>
       <c r="L15" s="3">
         <v>0</v>
       </c>
       <c r="M15" s="3">
-        <v>3</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <v>0</v>
       </c>
       <c r="O15" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Q15" s="3">
-        <v>3</v>
+      <c r="Q15" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="R15" s="3">
         <v>0</v>
       </c>
-      <c r="S15" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T15" s="3" t="s">
-        <v>19</v>
+      <c r="S15" s="3">
+        <v>0</v>
+      </c>
+      <c r="T15" s="3">
+        <v>3</v>
       </c>
       <c r="U15" s="3">
-        <v>3</v>
-      </c>
-      <c r="V15" s="3" t="s">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="V15" s="3">
+        <v>3</v>
       </c>
       <c r="W15" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X15" s="3">
         <v>0</v>
@@ -6485,14 +6507,14 @@
       <c r="Y15" s="3">
         <v>3</v>
       </c>
-      <c r="Z15" s="3">
-        <v>0</v>
+      <c r="Z15" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="AA15" s="3">
         <v>3</v>
       </c>
       <c r="AB15" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC15" s="3">
         <v>3</v>
@@ -6506,19 +6528,21 @@
       <c r="AF15" s="3">
         <v>0</v>
       </c>
-      <c r="AG15" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AH15" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AI15" s="3" t="s">
-        <v>19</v>
+      <c r="AG15" s="3">
+        <v>3</v>
+      </c>
+      <c r="AH15" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="3">
+        <v>0</v>
       </c>
       <c r="AJ15" s="3">
-        <v>3</v>
-      </c>
-      <c r="AK15" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="AK15" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL15" s="3"/>
       <c r="AM15" s="3"/>
       <c r="AN15" s="3"/>
@@ -6549,28 +6573,28 @@
         <v>17</v>
       </c>
       <c r="C16" s="6">
-        <f t="shared" si="2"/>
-        <v>12</v>
+        <f>SUM(I16:BI16)</f>
+        <v>15</v>
       </c>
       <c r="D16" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I16:V16)</f>
         <v>0</v>
       </c>
       <c r="E16" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W16:AI16)</f>
         <v>9</v>
       </c>
       <c r="F16" s="11">
-        <f t="shared" si="5"/>
-        <v>3</v>
+        <f>SUM(AJ16:AV16)</f>
+        <v>6</v>
       </c>
       <c r="G16" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW16:BI16)</f>
         <v>0</v>
       </c>
       <c r="H16" s="11">
-        <f t="shared" si="7"/>
-        <v>4</v>
+        <f>COUNT(I16:BI16)</f>
+        <v>5</v>
       </c>
       <c r="I16" s="3" t="s">
         <v>19</v>
@@ -6656,7 +6680,9 @@
       <c r="AJ16" s="3">
         <v>3</v>
       </c>
-      <c r="AK16" s="3"/>
+      <c r="AK16" s="3">
+        <v>3</v>
+      </c>
       <c r="AL16" s="3"/>
       <c r="AM16" s="3"/>
       <c r="AN16" s="3"/>
@@ -6687,27 +6713,27 @@
         <v>10</v>
       </c>
       <c r="C17" s="6">
-        <f t="shared" si="2"/>
+        <f>SUM(I17:BI17)</f>
         <v>1</v>
       </c>
       <c r="D17" s="11">
-        <f t="shared" si="3"/>
+        <f>SUM(I17:V17)</f>
         <v>1</v>
       </c>
       <c r="E17" s="11">
-        <f t="shared" si="4"/>
+        <f>SUM(W17:AI17)</f>
         <v>0</v>
       </c>
       <c r="F17" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(AJ17:AV17)</f>
         <v>0</v>
       </c>
       <c r="G17" s="11">
-        <f t="shared" si="6"/>
+        <f>SUM(AW17:BI17)</f>
         <v>0</v>
       </c>
       <c r="H17" s="11">
-        <f t="shared" si="7"/>
+        <f>COUNT(I17:BI17)</f>
         <v>2</v>
       </c>
       <c r="I17" s="3" t="s">
@@ -6794,7 +6820,9 @@
       <c r="AJ17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK17" s="3"/>
+      <c r="AK17" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL17" s="3"/>
       <c r="AM17" s="3"/>
       <c r="AN17" s="3"/>
@@ -6846,27 +6874,27 @@
         <v>46025</v>
       </c>
       <c r="J18" s="5">
-        <f t="shared" ref="J18:O18" si="8">I18+7</f>
+        <f t="shared" ref="J18:O18" si="2">I18+7</f>
         <v>46032</v>
       </c>
       <c r="K18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46039</v>
       </c>
       <c r="L18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46046</v>
       </c>
       <c r="M18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46053</v>
       </c>
       <c r="N18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46060</v>
       </c>
       <c r="O18" s="5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="2"/>
         <v>46067</v>
       </c>
       <c r="P18" s="5">
@@ -6897,159 +6925,159 @@
         <v>46109</v>
       </c>
       <c r="W18" s="5">
-        <f t="shared" ref="W18:BH18" si="9">V18+7</f>
+        <f t="shared" ref="W18:BH18" si="3">V18+7</f>
         <v>46116</v>
       </c>
       <c r="X18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46123</v>
       </c>
       <c r="Y18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46130</v>
       </c>
       <c r="Z18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46137</v>
       </c>
       <c r="AA18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46144</v>
       </c>
       <c r="AB18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46151</v>
       </c>
       <c r="AC18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46158</v>
       </c>
       <c r="AD18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46165</v>
       </c>
       <c r="AE18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46172</v>
       </c>
       <c r="AF18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46179</v>
       </c>
       <c r="AG18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46186</v>
       </c>
       <c r="AH18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46193</v>
       </c>
       <c r="AI18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46200</v>
       </c>
       <c r="AJ18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46207</v>
       </c>
       <c r="AK18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46214</v>
       </c>
       <c r="AL18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46221</v>
       </c>
       <c r="AM18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46228</v>
       </c>
       <c r="AN18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46235</v>
       </c>
       <c r="AO18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46242</v>
       </c>
       <c r="AP18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46249</v>
       </c>
       <c r="AQ18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46256</v>
       </c>
       <c r="AR18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46263</v>
       </c>
       <c r="AS18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46270</v>
       </c>
       <c r="AT18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46277</v>
       </c>
       <c r="AU18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46284</v>
       </c>
       <c r="AV18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46291</v>
       </c>
       <c r="AW18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46298</v>
       </c>
       <c r="AX18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46305</v>
       </c>
       <c r="AY18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46312</v>
       </c>
       <c r="AZ18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46319</v>
       </c>
       <c r="BA18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46326</v>
       </c>
       <c r="BB18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46333</v>
       </c>
       <c r="BC18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46340</v>
       </c>
       <c r="BD18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46347</v>
       </c>
       <c r="BE18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46354</v>
       </c>
       <c r="BF18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46361</v>
       </c>
       <c r="BG18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46368</v>
       </c>
       <c r="BH18" s="5">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>46375</v>
       </c>
       <c r="BI18" s="5">
-        <f t="shared" ref="BI18" si="10">BH18+7</f>
+        <f t="shared" ref="BI18" si="4">BH18+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -7079,7 +7107,7 @@
       </c>
       <c r="H19" s="11">
         <f>COUNT(I19:BI19)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I19" s="3">
         <v>3</v>
@@ -7165,7 +7193,9 @@
       <c r="AJ19" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK19" s="3"/>
+      <c r="AK19" s="3">
+        <v>0</v>
+      </c>
       <c r="AL19" s="3"/>
       <c r="AM19" s="3"/>
       <c r="AN19" s="3"/>
@@ -7197,7 +7227,7 @@
       </c>
       <c r="C20" s="6">
         <f>SUM(I20:BI20)</f>
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D20" s="11">
         <f>SUM(I20:V20)</f>
@@ -7209,7 +7239,7 @@
       </c>
       <c r="F20" s="11">
         <f>SUM(AJ20:AV20)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G20" s="11">
         <f>SUM(AW20:BI20)</f>
@@ -7217,7 +7247,7 @@
       </c>
       <c r="H20" s="11">
         <f>COUNT(I20:BI20)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>19</v>
@@ -7303,7 +7333,9 @@
       <c r="AJ20" s="3">
         <v>0</v>
       </c>
-      <c r="AK20" s="3"/>
+      <c r="AK20" s="3">
+        <v>3</v>
+      </c>
       <c r="AL20" s="3"/>
       <c r="AM20" s="3"/>
       <c r="AN20" s="3"/>
@@ -7423,23 +7455,23 @@
         <v>46032</v>
       </c>
       <c r="K23" s="5">
-        <f t="shared" ref="K23:BH23" si="11">J23+7</f>
+        <f t="shared" ref="K23:BH23" si="5">J23+7</f>
         <v>46039</v>
       </c>
       <c r="L23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46046</v>
       </c>
       <c r="M23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46053</v>
       </c>
       <c r="N23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46060</v>
       </c>
       <c r="O23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46067</v>
       </c>
       <c r="P23" s="5">
@@ -7450,179 +7482,179 @@
         <v>46074</v>
       </c>
       <c r="R23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46081</v>
       </c>
       <c r="S23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46088</v>
       </c>
       <c r="T23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46095</v>
       </c>
       <c r="U23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46102</v>
       </c>
       <c r="V23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46109</v>
       </c>
       <c r="W23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46116</v>
       </c>
       <c r="X23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46123</v>
       </c>
       <c r="Y23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46130</v>
       </c>
       <c r="Z23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46137</v>
       </c>
       <c r="AA23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46144</v>
       </c>
       <c r="AB23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46151</v>
       </c>
       <c r="AC23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46158</v>
       </c>
       <c r="AD23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46165</v>
       </c>
       <c r="AE23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46172</v>
       </c>
       <c r="AF23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46179</v>
       </c>
       <c r="AG23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46186</v>
       </c>
       <c r="AH23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46193</v>
       </c>
       <c r="AI23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46200</v>
       </c>
       <c r="AJ23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46207</v>
       </c>
       <c r="AK23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46214</v>
       </c>
       <c r="AL23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46221</v>
       </c>
       <c r="AM23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46228</v>
       </c>
       <c r="AN23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46235</v>
       </c>
       <c r="AO23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46242</v>
       </c>
       <c r="AP23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46249</v>
       </c>
       <c r="AQ23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46256</v>
       </c>
       <c r="AR23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46263</v>
       </c>
       <c r="AS23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46270</v>
       </c>
       <c r="AT23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46277</v>
       </c>
       <c r="AU23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46284</v>
       </c>
       <c r="AV23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46291</v>
       </c>
       <c r="AW23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46298</v>
       </c>
       <c r="AX23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46305</v>
       </c>
       <c r="AY23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46312</v>
       </c>
       <c r="AZ23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46319</v>
       </c>
       <c r="BA23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46326</v>
       </c>
       <c r="BB23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46333</v>
       </c>
       <c r="BC23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46340</v>
       </c>
       <c r="BD23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46347</v>
       </c>
       <c r="BE23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46354</v>
       </c>
       <c r="BF23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46361</v>
       </c>
       <c r="BG23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46368</v>
       </c>
       <c r="BH23" s="5">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>46375</v>
       </c>
       <c r="BI23" s="5">
-        <f t="shared" ref="BI23" si="12">BH23+7</f>
+        <f t="shared" ref="BI23" si="6">BH23+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -7631,28 +7663,28 @@
         <v>40</v>
       </c>
       <c r="C24" s="6">
-        <f t="shared" ref="C24:C37" si="13">SUM(I24:BI24)</f>
-        <v>44</v>
+        <f>SUM(I24:BI24)</f>
+        <v>45</v>
       </c>
       <c r="D24" s="11">
-        <f t="shared" ref="D24:D37" si="14">SUM(I24:V24)</f>
+        <f>SUM(I24:V24)</f>
         <v>20</v>
       </c>
       <c r="E24" s="11">
-        <f t="shared" ref="E24:E37" si="15">SUM(W24:AI24)</f>
+        <f>SUM(W24:AI24)</f>
         <v>24</v>
       </c>
       <c r="F24" s="11">
-        <f t="shared" ref="F24:F37" si="16">SUM(AJ24:AV24)</f>
-        <v>0</v>
+        <f>SUM(AJ24:AV24)</f>
+        <v>1</v>
       </c>
       <c r="G24" s="11">
-        <f t="shared" ref="G24:G37" si="17">SUM(AW24:BI24)</f>
+        <f>SUM(AW24:BI24)</f>
         <v>0</v>
       </c>
       <c r="H24" s="11">
-        <f t="shared" ref="H24:H37" si="18">COUNT(I24:BI24)</f>
-        <v>23</v>
+        <f>COUNT(I24:BI24)</f>
+        <v>24</v>
       </c>
       <c r="I24" s="3">
         <v>2</v>
@@ -7738,7 +7770,9 @@
       <c r="AJ24" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK24" s="3"/>
+      <c r="AK24" s="3">
+        <v>1</v>
+      </c>
       <c r="AL24" s="3"/>
       <c r="AM24" s="3"/>
       <c r="AN24" s="3"/>
@@ -7769,28 +7803,28 @@
         <v>9</v>
       </c>
       <c r="C25" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I25:BI25)</f>
         <v>40</v>
       </c>
       <c r="D25" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I25:V25)</f>
         <v>22</v>
       </c>
       <c r="E25" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W25:AI25)</f>
         <v>17</v>
       </c>
       <c r="F25" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ25:AV25)</f>
         <v>1</v>
       </c>
       <c r="G25" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW25:BI25)</f>
         <v>0</v>
       </c>
       <c r="H25" s="11">
-        <f t="shared" si="18"/>
-        <v>25</v>
+        <f>COUNT(I25:BI25)</f>
+        <v>26</v>
       </c>
       <c r="I25" s="3">
         <v>0</v>
@@ -7876,7 +7910,9 @@
       <c r="AJ25" s="3">
         <v>1</v>
       </c>
-      <c r="AK25" s="3"/>
+      <c r="AK25" s="3">
+        <v>0</v>
+      </c>
       <c r="AL25" s="3"/>
       <c r="AM25" s="3"/>
       <c r="AN25" s="3"/>
@@ -7904,109 +7940,109 @@
     </row>
     <row r="26" spans="2:61" ht="14.1" customHeight="1">
       <c r="B26" s="14" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C26" s="6">
-        <f t="shared" si="13"/>
-        <v>35</v>
+        <f>SUM(I26:BI26)</f>
+        <v>36</v>
       </c>
       <c r="D26" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I26:V26)</f>
         <v>19</v>
       </c>
       <c r="E26" s="11">
-        <f t="shared" si="15"/>
-        <v>15</v>
+        <f>SUM(W26:AI26)</f>
+        <v>12</v>
       </c>
       <c r="F26" s="11">
-        <f t="shared" si="16"/>
-        <v>1</v>
+        <f>SUM(AJ26:AV26)</f>
+        <v>5</v>
       </c>
       <c r="G26" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW26:BI26)</f>
         <v>0</v>
       </c>
       <c r="H26" s="11">
-        <f t="shared" si="18"/>
-        <v>23</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>19</v>
+        <f>COUNT(I26:BI26)</f>
+        <v>25</v>
+      </c>
+      <c r="I26" s="3">
+        <v>4</v>
       </c>
       <c r="J26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M26" s="3">
-        <v>3</v>
-      </c>
-      <c r="N26" s="3">
+        <v>1</v>
+      </c>
+      <c r="N26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O26" s="3">
+        <v>3</v>
+      </c>
+      <c r="P26" s="3">
         <v>2</v>
       </c>
-      <c r="O26" s="3">
+      <c r="Q26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R26" s="3">
+        <v>1</v>
+      </c>
+      <c r="S26" s="3">
         <v>2</v>
       </c>
-      <c r="P26" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="3">
+      <c r="T26" s="3">
+        <v>0</v>
+      </c>
+      <c r="U26" s="3">
+        <v>1</v>
+      </c>
+      <c r="V26" s="3">
+        <v>1</v>
+      </c>
+      <c r="W26" s="3">
+        <v>0</v>
+      </c>
+      <c r="X26" s="3">
+        <v>3</v>
+      </c>
+      <c r="Y26" s="3">
+        <v>3</v>
+      </c>
+      <c r="Z26" s="3">
+        <v>1</v>
+      </c>
+      <c r="AA26" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AC26" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD26" s="3">
         <v>2</v>
       </c>
-      <c r="R26" s="3">
-        <v>1</v>
-      </c>
-      <c r="S26" s="3">
-        <v>1</v>
-      </c>
-      <c r="T26" s="3">
-        <v>1</v>
-      </c>
-      <c r="U26" s="3">
-        <v>1</v>
-      </c>
-      <c r="V26" s="3">
-        <v>2</v>
-      </c>
-      <c r="W26" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="X26" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y26" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="Z26" s="3">
-        <v>3</v>
-      </c>
-      <c r="AA26" s="3">
-        <v>2</v>
-      </c>
-      <c r="AB26" s="3">
-        <v>5</v>
-      </c>
-      <c r="AC26" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD26" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AE26" s="3" t="s">
-        <v>19</v>
+      <c r="AE26" s="3">
+        <v>1</v>
       </c>
       <c r="AF26" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG26" s="3">
         <v>0</v>
       </c>
       <c r="AH26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI26" s="3">
         <v>1</v>
@@ -8014,7 +8050,9 @@
       <c r="AJ26" s="3">
         <v>1</v>
       </c>
-      <c r="AK26" s="3"/>
+      <c r="AK26" s="3">
+        <v>4</v>
+      </c>
       <c r="AL26" s="3"/>
       <c r="AM26" s="3"/>
       <c r="AN26" s="3"/>
@@ -8042,109 +8080,109 @@
     </row>
     <row r="27" spans="2:61" ht="14.1" customHeight="1">
       <c r="B27" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="6">
+        <f>SUM(I27:BI27)</f>
+        <v>35</v>
+      </c>
+      <c r="D27" s="11">
+        <f>SUM(I27:V27)</f>
+        <v>19</v>
+      </c>
+      <c r="E27" s="11">
+        <f>SUM(W27:AI27)</f>
+        <v>15</v>
+      </c>
+      <c r="F27" s="11">
+        <f>SUM(AJ27:AV27)</f>
+        <v>1</v>
+      </c>
+      <c r="G27" s="11">
+        <f>SUM(AW27:BI27)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="11">
+        <f>COUNT(I27:BI27)</f>
+        <v>24</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J27" s="3">
+        <v>0</v>
+      </c>
+      <c r="K27" s="3">
+        <v>3</v>
+      </c>
+      <c r="L27" s="3">
+        <v>0</v>
+      </c>
+      <c r="M27" s="3">
+        <v>3</v>
+      </c>
+      <c r="N27" s="3">
+        <v>2</v>
+      </c>
+      <c r="O27" s="3">
+        <v>2</v>
+      </c>
+      <c r="P27" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>2</v>
+      </c>
+      <c r="R27" s="3">
+        <v>1</v>
+      </c>
+      <c r="S27" s="3">
+        <v>1</v>
+      </c>
+      <c r="T27" s="3">
+        <v>1</v>
+      </c>
+      <c r="U27" s="3">
+        <v>1</v>
+      </c>
+      <c r="V27" s="3">
+        <v>2</v>
+      </c>
+      <c r="W27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="X27" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Z27" s="3">
+        <v>3</v>
+      </c>
+      <c r="AA27" s="3">
+        <v>2</v>
+      </c>
+      <c r="AB27" s="3">
         <v>5</v>
       </c>
-      <c r="C27" s="6">
-        <f t="shared" si="13"/>
-        <v>32</v>
-      </c>
-      <c r="D27" s="11">
-        <f t="shared" si="14"/>
-        <v>19</v>
-      </c>
-      <c r="E27" s="11">
-        <f t="shared" si="15"/>
-        <v>12</v>
-      </c>
-      <c r="F27" s="11">
-        <f t="shared" si="16"/>
-        <v>1</v>
-      </c>
-      <c r="G27" s="11">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="H27" s="11">
-        <f t="shared" si="18"/>
-        <v>24</v>
-      </c>
-      <c r="I27" s="3">
-        <v>4</v>
-      </c>
-      <c r="J27" s="3">
-        <v>1</v>
-      </c>
-      <c r="K27" s="3">
+      <c r="AC27" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE27" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="AF27" s="3">
         <v>2</v>
       </c>
-      <c r="L27" s="3">
-        <v>1</v>
-      </c>
-      <c r="M27" s="3">
-        <v>1</v>
-      </c>
-      <c r="N27" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="O27" s="3">
-        <v>3</v>
-      </c>
-      <c r="P27" s="3">
-        <v>2</v>
-      </c>
-      <c r="Q27" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="R27" s="3">
-        <v>1</v>
-      </c>
-      <c r="S27" s="3">
-        <v>2</v>
-      </c>
-      <c r="T27" s="3">
-        <v>0</v>
-      </c>
-      <c r="U27" s="3">
-        <v>1</v>
-      </c>
-      <c r="V27" s="3">
-        <v>1</v>
-      </c>
-      <c r="W27" s="3">
-        <v>0</v>
-      </c>
-      <c r="X27" s="3">
-        <v>3</v>
-      </c>
-      <c r="Y27" s="3">
-        <v>3</v>
-      </c>
-      <c r="Z27" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA27" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB27" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AC27" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="AD27" s="3">
-        <v>2</v>
-      </c>
-      <c r="AE27" s="3">
-        <v>1</v>
-      </c>
-      <c r="AF27" s="3">
-        <v>1</v>
-      </c>
       <c r="AG27" s="3">
         <v>0</v>
       </c>
       <c r="AH27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI27" s="3">
         <v>1</v>
@@ -8152,7 +8190,9 @@
       <c r="AJ27" s="3">
         <v>1</v>
       </c>
-      <c r="AK27" s="3"/>
+      <c r="AK27" s="3">
+        <v>0</v>
+      </c>
       <c r="AL27" s="3"/>
       <c r="AM27" s="3"/>
       <c r="AN27" s="3"/>
@@ -8183,28 +8223,28 @@
         <v>11</v>
       </c>
       <c r="C28" s="6">
-        <f t="shared" si="13"/>
-        <v>28</v>
+        <f>SUM(I28:BI28)</f>
+        <v>29</v>
       </c>
       <c r="D28" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I28:V28)</f>
         <v>14</v>
       </c>
       <c r="E28" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W28:AI28)</f>
         <v>14</v>
       </c>
       <c r="F28" s="11">
-        <f t="shared" si="16"/>
-        <v>0</v>
+        <f>SUM(AJ28:AV28)</f>
+        <v>1</v>
       </c>
       <c r="G28" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW28:BI28)</f>
         <v>0</v>
       </c>
       <c r="H28" s="11">
-        <f t="shared" si="18"/>
-        <v>20</v>
+        <f>COUNT(I28:BI28)</f>
+        <v>21</v>
       </c>
       <c r="I28" s="3">
         <v>0</v>
@@ -8290,7 +8330,9 @@
       <c r="AJ28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK28" s="3"/>
+      <c r="AK28" s="3">
+        <v>1</v>
+      </c>
       <c r="AL28" s="3"/>
       <c r="AM28" s="3"/>
       <c r="AN28" s="3"/>
@@ -8321,27 +8363,27 @@
         <v>3</v>
       </c>
       <c r="C29" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I29:BI29)</f>
         <v>28</v>
       </c>
       <c r="D29" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I29:V29)</f>
         <v>10</v>
       </c>
       <c r="E29" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W29:AI29)</f>
         <v>17</v>
       </c>
       <c r="F29" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ29:AV29)</f>
         <v>1</v>
       </c>
       <c r="G29" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW29:BI29)</f>
         <v>0</v>
       </c>
       <c r="H29" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I29:BI29)</f>
         <v>24</v>
       </c>
       <c r="I29" s="3">
@@ -8428,7 +8470,9 @@
       <c r="AJ29" s="3">
         <v>1</v>
       </c>
-      <c r="AK29" s="3"/>
+      <c r="AK29" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL29" s="3"/>
       <c r="AM29" s="3"/>
       <c r="AN29" s="3"/>
@@ -8456,34 +8500,34 @@
     </row>
     <row r="30" spans="2:61" ht="14.1" customHeight="1">
       <c r="B30" s="14" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="C30" s="6">
-        <f t="shared" si="13"/>
-        <v>23</v>
+        <f>SUM(I30:BI30)</f>
+        <v>24</v>
       </c>
       <c r="D30" s="11">
-        <f t="shared" si="14"/>
-        <v>13</v>
+        <f>SUM(I30:V30)</f>
+        <v>11</v>
       </c>
       <c r="E30" s="11">
-        <f t="shared" si="15"/>
-        <v>10</v>
+        <f>SUM(W30:AI30)</f>
+        <v>12</v>
       </c>
       <c r="F30" s="11">
-        <f t="shared" si="16"/>
-        <v>0</v>
+        <f>SUM(AJ30:AV30)</f>
+        <v>1</v>
       </c>
       <c r="G30" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW30:BI30)</f>
         <v>0</v>
       </c>
       <c r="H30" s="11">
-        <f t="shared" si="18"/>
-        <v>26</v>
+        <f>COUNT(I30:BI30)</f>
+        <v>28</v>
       </c>
       <c r="I30" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J30" s="3">
         <v>0</v>
@@ -8492,55 +8536,55 @@
         <v>0</v>
       </c>
       <c r="L30" s="3">
-        <v>0</v>
-      </c>
-      <c r="M30" s="3" t="s">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="M30" s="3">
+        <v>0</v>
       </c>
       <c r="N30" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O30" s="3">
-        <v>5</v>
-      </c>
-      <c r="P30" s="3" t="s">
-        <v>19</v>
+        <v>1</v>
+      </c>
+      <c r="P30" s="3">
+        <v>0</v>
       </c>
       <c r="Q30" s="3">
+        <v>0</v>
+      </c>
+      <c r="R30" s="3">
+        <v>1</v>
+      </c>
+      <c r="S30" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T30" s="3">
+        <v>1</v>
+      </c>
+      <c r="U30" s="3">
+        <v>1</v>
+      </c>
+      <c r="V30" s="3">
         <v>2</v>
       </c>
-      <c r="R30" s="3">
-        <v>0</v>
-      </c>
-      <c r="S30" s="3">
-        <v>1</v>
-      </c>
-      <c r="T30" s="3">
+      <c r="W30" s="3">
+        <v>0</v>
+      </c>
+      <c r="X30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="3">
         <v>2</v>
       </c>
-      <c r="U30" s="3">
-        <v>3</v>
-      </c>
-      <c r="V30" s="3">
-        <v>0</v>
-      </c>
-      <c r="W30" s="3">
-        <v>1</v>
-      </c>
-      <c r="X30" s="3">
-        <v>1</v>
-      </c>
-      <c r="Y30" s="3">
-        <v>2</v>
-      </c>
-      <c r="Z30" s="3">
-        <v>0</v>
-      </c>
       <c r="AA30" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB30" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AC30" s="3">
         <v>1</v>
@@ -8552,21 +8596,23 @@
         <v>0</v>
       </c>
       <c r="AF30" s="3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AG30" s="3">
         <v>2</v>
       </c>
       <c r="AH30" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AI30" s="3">
         <v>0</v>
       </c>
       <c r="AJ30" s="3">
-        <v>0</v>
-      </c>
-      <c r="AK30" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="AK30" s="3">
+        <v>0</v>
+      </c>
       <c r="AL30" s="3"/>
       <c r="AM30" s="3"/>
       <c r="AN30" s="3"/>
@@ -8594,92 +8640,92 @@
     </row>
     <row r="31" spans="2:61" ht="14.1" customHeight="1">
       <c r="B31" s="14" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="C31" s="6">
-        <f t="shared" si="13"/>
-        <v>24</v>
+        <f>SUM(I31:BI31)</f>
+        <v>23</v>
       </c>
       <c r="D31" s="11">
-        <f t="shared" si="14"/>
-        <v>11</v>
+        <f>SUM(I31:V31)</f>
+        <v>13</v>
       </c>
       <c r="E31" s="11">
-        <f t="shared" si="15"/>
-        <v>12</v>
+        <f>SUM(W31:AI31)</f>
+        <v>10</v>
       </c>
       <c r="F31" s="11">
-        <f t="shared" si="16"/>
-        <v>1</v>
+        <f>SUM(AJ31:AV31)</f>
+        <v>0</v>
       </c>
       <c r="G31" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW31:BI31)</f>
         <v>0</v>
       </c>
       <c r="H31" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I31:BI31)</f>
         <v>27</v>
       </c>
       <c r="I31" s="3">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3">
+        <v>0</v>
+      </c>
+      <c r="L31" s="3">
+        <v>0</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N31" s="3">
+        <v>0</v>
+      </c>
+      <c r="O31" s="3">
+        <v>5</v>
+      </c>
+      <c r="P31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q31" s="3">
         <v>2</v>
       </c>
-      <c r="J31" s="3">
-        <v>0</v>
-      </c>
-      <c r="K31" s="3">
-        <v>0</v>
-      </c>
-      <c r="L31" s="3">
-        <v>1</v>
-      </c>
-      <c r="M31" s="3">
-        <v>0</v>
-      </c>
-      <c r="N31" s="3">
+      <c r="R31" s="3">
+        <v>0</v>
+      </c>
+      <c r="S31" s="3">
+        <v>1</v>
+      </c>
+      <c r="T31" s="3">
         <v>2</v>
       </c>
-      <c r="O31" s="3">
-        <v>1</v>
-      </c>
-      <c r="P31" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="3">
-        <v>0</v>
-      </c>
-      <c r="R31" s="3">
-        <v>1</v>
-      </c>
-      <c r="S31" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="T31" s="3">
-        <v>1</v>
-      </c>
       <c r="U31" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V31" s="3">
+        <v>0</v>
+      </c>
+      <c r="W31" s="3">
+        <v>1</v>
+      </c>
+      <c r="X31" s="3">
+        <v>1</v>
+      </c>
+      <c r="Y31" s="3">
         <v>2</v>
       </c>
-      <c r="W31" s="3">
-        <v>0</v>
-      </c>
-      <c r="X31" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y31" s="3">
-        <v>0</v>
-      </c>
       <c r="Z31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="3">
         <v>2</v>
       </c>
-      <c r="AA31" s="3">
-        <v>1</v>
-      </c>
-      <c r="AB31" s="3">
-        <v>0</v>
-      </c>
       <c r="AC31" s="3">
         <v>1</v>
       </c>
@@ -8690,21 +8736,23 @@
         <v>0</v>
       </c>
       <c r="AF31" s="3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AG31" s="3">
         <v>2</v>
       </c>
       <c r="AH31" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AI31" s="3">
         <v>0</v>
       </c>
       <c r="AJ31" s="3">
-        <v>1</v>
-      </c>
-      <c r="AK31" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="AK31" s="3">
+        <v>0</v>
+      </c>
       <c r="AL31" s="3"/>
       <c r="AM31" s="3"/>
       <c r="AN31" s="3"/>
@@ -8735,27 +8783,27 @@
         <v>15</v>
       </c>
       <c r="C32" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I32:BI32)</f>
         <v>19</v>
       </c>
       <c r="D32" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I32:V32)</f>
         <v>8</v>
       </c>
       <c r="E32" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W32:AI32)</f>
         <v>11</v>
       </c>
       <c r="F32" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ32:AV32)</f>
         <v>0</v>
       </c>
       <c r="G32" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW32:BI32)</f>
         <v>0</v>
       </c>
       <c r="H32" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I32:BI32)</f>
         <v>14</v>
       </c>
       <c r="I32" s="3" t="s">
@@ -8842,7 +8890,9 @@
       <c r="AJ32" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK32" s="3"/>
+      <c r="AK32" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL32" s="3"/>
       <c r="AM32" s="3"/>
       <c r="AN32" s="3"/>
@@ -8873,28 +8923,28 @@
         <v>7</v>
       </c>
       <c r="C33" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I33:BI33)</f>
         <v>16</v>
       </c>
       <c r="D33" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I33:V33)</f>
         <v>10</v>
       </c>
       <c r="E33" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W33:AI33)</f>
         <v>6</v>
       </c>
       <c r="F33" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ33:AV33)</f>
         <v>0</v>
       </c>
       <c r="G33" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW33:BI33)</f>
         <v>0</v>
       </c>
       <c r="H33" s="11">
-        <f t="shared" si="18"/>
-        <v>20</v>
+        <f>COUNT(I33:BI33)</f>
+        <v>21</v>
       </c>
       <c r="I33" s="3">
         <v>2</v>
@@ -8980,7 +9030,9 @@
       <c r="AJ33" s="3">
         <v>0</v>
       </c>
-      <c r="AK33" s="3"/>
+      <c r="AK33" s="3">
+        <v>0</v>
+      </c>
       <c r="AL33" s="3"/>
       <c r="AM33" s="3"/>
       <c r="AN33" s="3"/>
@@ -9011,28 +9063,28 @@
         <v>6</v>
       </c>
       <c r="C34" s="6">
-        <f t="shared" si="13"/>
-        <v>8</v>
+        <f>SUM(I34:BI34)</f>
+        <v>10</v>
       </c>
       <c r="D34" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I34:V34)</f>
         <v>4</v>
       </c>
       <c r="E34" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W34:AI34)</f>
         <v>3</v>
       </c>
       <c r="F34" s="11">
-        <f t="shared" si="16"/>
-        <v>1</v>
+        <f>SUM(AJ34:AV34)</f>
+        <v>3</v>
       </c>
       <c r="G34" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW34:BI34)</f>
         <v>0</v>
       </c>
       <c r="H34" s="11">
-        <f t="shared" si="18"/>
-        <v>17</v>
+        <f>COUNT(I34:BI34)</f>
+        <v>18</v>
       </c>
       <c r="I34" s="3">
         <v>0</v>
@@ -9118,7 +9170,9 @@
       <c r="AJ34" s="3">
         <v>1</v>
       </c>
-      <c r="AK34" s="3"/>
+      <c r="AK34" s="3">
+        <v>2</v>
+      </c>
       <c r="AL34" s="3"/>
       <c r="AM34" s="3"/>
       <c r="AN34" s="3"/>
@@ -9149,28 +9203,28 @@
         <v>36</v>
       </c>
       <c r="C35" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I35:BI35)</f>
         <v>5</v>
       </c>
       <c r="D35" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I35:V35)</f>
         <v>3</v>
       </c>
       <c r="E35" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W35:AI35)</f>
         <v>2</v>
       </c>
       <c r="F35" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ35:AV35)</f>
         <v>0</v>
       </c>
       <c r="G35" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW35:BI35)</f>
         <v>0</v>
       </c>
       <c r="H35" s="11">
-        <f t="shared" si="18"/>
-        <v>17</v>
+        <f>COUNT(I35:BI35)</f>
+        <v>18</v>
       </c>
       <c r="I35" s="3" t="s">
         <v>19</v>
@@ -9256,7 +9310,9 @@
       <c r="AJ35" s="3">
         <v>0</v>
       </c>
-      <c r="AK35" s="3"/>
+      <c r="AK35" s="3">
+        <v>0</v>
+      </c>
       <c r="AL35" s="3"/>
       <c r="AM35" s="3"/>
       <c r="AN35" s="3"/>
@@ -9287,28 +9343,28 @@
         <v>17</v>
       </c>
       <c r="C36" s="6">
-        <f t="shared" si="13"/>
-        <v>3</v>
+        <f>SUM(I36:BI36)</f>
+        <v>4</v>
       </c>
       <c r="D36" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I36:V36)</f>
         <v>0</v>
       </c>
       <c r="E36" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W36:AI36)</f>
         <v>3</v>
       </c>
       <c r="F36" s="11">
-        <f t="shared" si="16"/>
-        <v>0</v>
+        <f>SUM(AJ36:AV36)</f>
+        <v>1</v>
       </c>
       <c r="G36" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW36:BI36)</f>
         <v>0</v>
       </c>
       <c r="H36" s="11">
-        <f t="shared" si="18"/>
-        <v>5</v>
+        <f>COUNT(I36:BI36)</f>
+        <v>6</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>19</v>
@@ -9394,7 +9450,9 @@
       <c r="AJ36" s="3">
         <v>0</v>
       </c>
-      <c r="AK36" s="3"/>
+      <c r="AK36" s="3">
+        <v>1</v>
+      </c>
       <c r="AL36" s="3"/>
       <c r="AM36" s="3"/>
       <c r="AN36" s="3"/>
@@ -9425,27 +9483,27 @@
         <v>10</v>
       </c>
       <c r="C37" s="6">
-        <f t="shared" si="13"/>
+        <f>SUM(I37:BI37)</f>
         <v>0</v>
       </c>
       <c r="D37" s="11">
-        <f t="shared" si="14"/>
+        <f>SUM(I37:V37)</f>
         <v>0</v>
       </c>
       <c r="E37" s="11">
-        <f t="shared" si="15"/>
+        <f>SUM(W37:AI37)</f>
         <v>0</v>
       </c>
       <c r="F37" s="11">
-        <f t="shared" si="16"/>
+        <f>SUM(AJ37:AV37)</f>
         <v>0</v>
       </c>
       <c r="G37" s="11">
-        <f t="shared" si="17"/>
+        <f>SUM(AW37:BI37)</f>
         <v>0</v>
       </c>
       <c r="H37" s="11">
-        <f t="shared" si="18"/>
+        <f>COUNT(I37:BI37)</f>
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
@@ -9532,7 +9590,9 @@
       <c r="AJ37" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="AK37" s="3"/>
+      <c r="AK37" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="AL37" s="3"/>
       <c r="AM37" s="3"/>
       <c r="AN37" s="3"/>
@@ -9588,23 +9648,23 @@
         <v>46032</v>
       </c>
       <c r="K38" s="5">
-        <f t="shared" ref="K38:BH38" si="19">J38+7</f>
+        <f t="shared" ref="K38:BH38" si="7">J38+7</f>
         <v>46039</v>
       </c>
       <c r="L38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46046</v>
       </c>
       <c r="M38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46053</v>
       </c>
       <c r="N38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46060</v>
       </c>
       <c r="O38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46067</v>
       </c>
       <c r="P38" s="5">
@@ -9615,179 +9675,179 @@
         <v>46074</v>
       </c>
       <c r="R38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46081</v>
       </c>
       <c r="S38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46088</v>
       </c>
       <c r="T38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46095</v>
       </c>
       <c r="U38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46102</v>
       </c>
       <c r="V38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46109</v>
       </c>
       <c r="W38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46116</v>
       </c>
       <c r="X38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46123</v>
       </c>
       <c r="Y38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46130</v>
       </c>
       <c r="Z38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46137</v>
       </c>
       <c r="AA38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46144</v>
       </c>
       <c r="AB38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46151</v>
       </c>
       <c r="AC38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46158</v>
       </c>
       <c r="AD38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46165</v>
       </c>
       <c r="AE38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46172</v>
       </c>
       <c r="AF38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46179</v>
       </c>
       <c r="AG38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46186</v>
       </c>
       <c r="AH38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46193</v>
       </c>
       <c r="AI38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46200</v>
       </c>
       <c r="AJ38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46207</v>
       </c>
       <c r="AK38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46214</v>
       </c>
       <c r="AL38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46221</v>
       </c>
       <c r="AM38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46228</v>
       </c>
       <c r="AN38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46235</v>
       </c>
       <c r="AO38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46242</v>
       </c>
       <c r="AP38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46249</v>
       </c>
       <c r="AQ38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46256</v>
       </c>
       <c r="AR38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46263</v>
       </c>
       <c r="AS38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46270</v>
       </c>
       <c r="AT38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46277</v>
       </c>
       <c r="AU38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46284</v>
       </c>
       <c r="AV38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46291</v>
       </c>
       <c r="AW38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46298</v>
       </c>
       <c r="AX38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46305</v>
       </c>
       <c r="AY38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46312</v>
       </c>
       <c r="AZ38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46319</v>
       </c>
       <c r="BA38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46326</v>
       </c>
       <c r="BB38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46333</v>
       </c>
       <c r="BC38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46340</v>
       </c>
       <c r="BD38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46347</v>
       </c>
       <c r="BE38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46354</v>
       </c>
       <c r="BF38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46361</v>
       </c>
       <c r="BG38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46368</v>
       </c>
       <c r="BH38" s="5">
-        <f t="shared" si="19"/>
+        <f t="shared" si="7"/>
         <v>46375</v>
       </c>
       <c r="BI38" s="5">
-        <f t="shared" ref="BI38" si="20">BH38+7</f>
+        <f t="shared" ref="BI38" si="8">BH38+7</f>
         <v>46382</v>
       </c>
     </row>
@@ -9800,24 +9860,24 @@
         <v>0</v>
       </c>
       <c r="D39" s="11">
-        <f t="shared" ref="D39:D40" si="21">SUM(I39:V39)</f>
+        <f t="shared" ref="D39:D40" si="9">SUM(I39:V39)</f>
         <v>0</v>
       </c>
       <c r="E39" s="11">
-        <f t="shared" ref="E39:E40" si="22">SUM(W39:AI39)</f>
+        <f t="shared" ref="E39:E40" si="10">SUM(W39:AI39)</f>
         <v>0</v>
       </c>
       <c r="F39" s="11">
-        <f t="shared" ref="F39:F40" si="23">SUM(AJ39:AV39)</f>
+        <f t="shared" ref="F39:F40" si="11">SUM(AJ39:AV39)</f>
         <v>0</v>
       </c>
       <c r="G39" s="11">
-        <f t="shared" ref="G39:G40" si="24">SUM(AW39:BI39)</f>
+        <f t="shared" ref="G39:G40" si="12">SUM(AW39:BI39)</f>
         <v>0</v>
       </c>
       <c r="H39" s="11">
-        <f t="shared" ref="H39:H40" si="25">COUNT(I39:BI39)</f>
-        <v>23</v>
+        <f t="shared" ref="H39:H40" si="13">COUNT(I39:BI39)</f>
+        <v>24</v>
       </c>
       <c r="I39" s="3">
         <v>0</v>
@@ -9903,7 +9963,9 @@
       <c r="AJ39" s="3">
         <v>0</v>
       </c>
-      <c r="AK39" s="3"/>
+      <c r="AK39" s="3">
+        <v>0</v>
+      </c>
       <c r="AL39" s="3"/>
       <c r="AM39" s="3"/>
       <c r="AN39" s="3"/>
@@ -9938,24 +10000,24 @@
         <v>0</v>
       </c>
       <c r="D40" s="11">
-        <f t="shared" si="21"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="E40" s="11">
-        <f t="shared" si="22"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F40" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="G40" s="11">
-        <f t="shared" si="24"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="H40" s="11">
-        <f t="shared" si="25"/>
-        <v>21</v>
+        <f t="shared" si="13"/>
+        <v>22</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>19</v>
@@ -10041,7 +10103,9 @@
       <c r="AJ40" s="3">
         <v>0</v>
       </c>
-      <c r="AK40" s="3"/>
+      <c r="AK40" s="3">
+        <v>0</v>
+      </c>
       <c r="AL40" s="3"/>
       <c r="AM40" s="3"/>
       <c r="AN40" s="3"/>
@@ -10068,8 +10132,8 @@
       <c r="BI40" s="3"/>
     </row>
   </sheetData>
-  <sortState ref="B4:AI17">
-    <sortCondition descending="1" ref="C4:C17"/>
+  <sortState ref="B24:AV37">
+    <sortCondition descending="1" ref="C24:C37"/>
   </sortState>
   <mergeCells count="2">
     <mergeCell ref="B22:BI22"/>
@@ -10078,7 +10142,7 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="E19:E20 F19:F20 E38:E40 E24:F37 F38:F40 F18 E18 E4:F17" formulaRange="1"/>
+    <ignoredError sqref="E19:E20 F19:F20 E38:E40 F38:F40 F18 E18 E5:F16 D25:F36" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>